<commit_message>
Commentless GitLatch Commit @ 2025-4-8-18-6-13-591
</commit_message>
<xml_diff>
--- a/excel_portfolioproject.xlsx
+++ b/excel_portfolioproject.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yedur\OneDrive\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{3C9CB034-3682-47AA-BF1C-9F007481A80A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{45669DD3-6796-465F-B026-43BDCD7286F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{26D4546B-D2A1-4444-8EAF-A6228F96F0C1}"/>
   </bookViews>
@@ -4279,7 +4279,7 @@
 </file>
 
 <file path=xl/webextensions/webextension1.xml><?xml version="1.0" encoding="utf-8"?>
-<we:webextension xmlns:we="http://schemas.microsoft.com/office/webextensions/webextension/2010/11" id="{768D9F54-A6D1-479A-BDA7-33E8DE7A3AA0}">
+<we:webextension xmlns:we="http://schemas.microsoft.com/office/webextensions/webextension/2010/11" id="{09726214-8154-41F4-8F67-0F6B56ED0881}">
   <we:reference id="wa200005069" version="1.0.0.3" store="en-US" storeType="OMEX"/>
   <we:alternateReferences>
     <we:reference id="wa200005069" version="1.0.0.3" store="wa200005069" storeType="OMEX"/>
@@ -43550,10 +43550,9 @@
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
   <tableParts count="2">
+    <tablePart r:id="rId1"/>
     <tablePart r:id="rId2"/>
-    <tablePart r:id="rId3"/>
   </tableParts>
 </worksheet>
 </file>
@@ -43617,7 +43616,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
-  <drawing r:id="rId2"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Commentless GitLatch Commit @ 2025-4-9-7-14-32-788
</commit_message>
<xml_diff>
--- a/excel_portfolioproject.xlsx
+++ b/excel_portfolioproject.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yedur\OneDrive\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B000F1F4-6394-4F23-ADF6-3C68E92867FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{C6D4327D-4D48-40E2-A694-33F74B9AEF32}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{26D4546B-D2A1-4444-8EAF-A6228F96F0C1}"/>
   </bookViews>
@@ -3834,7 +3834,7 @@
     </mc:Fallback>
   </mc:AlternateContent>
   <c:pivotSource>
-    <c:name>[excel_portfolioproject.xlsx]pivot!PivotTable4</c:name>
+    <c:name>[excel_portfolioproject.xlsx]pivot!weekly trend</c:name>
     <c:fmtId val="17"/>
   </c:pivotSource>
   <c:chart>
@@ -9266,7 +9266,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{AAB53815-8D20-4469-8EC4-4352A86443FA}" name="PivotTable4" cacheId="3" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" subtotalHiddenItems="1" itemPrintTitles="1" createdVersion="8" indent="0" multipleFieldFilters="0" chartFormat="23">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{AAB53815-8D20-4469-8EC4-4352A86443FA}" name="weekly trend" cacheId="3" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" subtotalHiddenItems="1" itemPrintTitles="1" createdVersion="8" indent="0" multipleFieldFilters="0" chartFormat="23">
   <location ref="E19:F27" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="3">
     <pivotField allDrilled="1" showAll="0" dataSourceSort="1" defaultAttributeDrillState="1"/>
@@ -9725,7 +9725,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{2C89DBDB-5792-4DE1-B0D8-F6BE6B3A85F2}" name="PivotTable2" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" subtotalHiddenItems="1" itemPrintTitles="1" createdVersion="8" indent="0" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{2C89DBDB-5792-4DE1-B0D8-F6BE6B3A85F2}" name="rep pivot" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" subtotalHiddenItems="1" itemPrintTitles="1" createdVersion="8" indent="0" multipleFieldFilters="0">
   <location ref="A11:E12" firstHeaderRow="0" firstDataRow="1" firstDataCol="0"/>
   <pivotFields count="6">
     <pivotField dataField="1" showAll="0"/>
@@ -9818,7 +9818,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{88456301-C695-4DCF-807F-7BCA00D1AD0A}" name="PivotTable1" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{88456301-C695-4DCF-807F-7BCA00D1AD0A}" name="summary pivot" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" multipleFieldFilters="0">
   <location ref="A3:E4" firstHeaderRow="0" firstDataRow="1" firstDataCol="0"/>
   <pivotFields count="5">
     <pivotField dataField="1" showAll="0"/>
@@ -9943,9 +9943,9 @@
 <file path=xl/slicerCaches/slicerCache1.xml><?xml version="1.0" encoding="utf-8"?>
 <slicerCacheDefinition xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x xr10" name="Slicer_Representative" xr10:uid="{6D395BF4-332F-4A8E-8EA8-129093CB3236}" sourceName="[calls].[Representative]">
   <pivotTables>
-    <pivotTable tabId="6" name="PivotTable2"/>
+    <pivotTable tabId="6" name="rep pivot"/>
     <pivotTable tabId="6" name="month trend"/>
-    <pivotTable tabId="6" name="PivotTable4"/>
+    <pivotTable tabId="6" name="weekly trend"/>
   </pivotTables>
   <data>
     <olap pivotCacheId="562902582">

</xml_diff>

<commit_message>
Commentless GitLatch Commit @ 2025-4-9-13-50-1-525
</commit_message>
<xml_diff>
--- a/excel_portfolioproject.xlsx
+++ b/excel_portfolioproject.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yedur\OneDrive\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{95222239-0A25-4591-87AF-4CD6EFB8FA38}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{F7264FCA-5584-451A-995B-8834A4525ECC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{26D4546B-D2A1-4444-8EAF-A6228F96F0C1}"/>
   </bookViews>
@@ -21,8 +21,8 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">Data!$B$3:$H$1003</definedName>
-    <definedName name="_xlcn.WorksheetConnection_excel_portfolioproject.xlsxcalls" hidden="1">calls[]</definedName>
-    <definedName name="_xlcn.WorksheetConnection_excel_portfolioproject.xlsxcustomers" hidden="1">customers[]</definedName>
+    <definedName name="_xlcn.WorksheetConnection_excel_portfolioproject.xlsxcalls1" hidden="1">calls[]</definedName>
+    <definedName name="_xlcn.WorksheetConnection_excel_portfolioproject.xlsxcustomers1" hidden="1">customers[]</definedName>
     <definedName name="ExternalData_1" localSheetId="0" hidden="1">Sheet1!$A$3:$K$221</definedName>
     <definedName name="Rep_pivot">pivot!$A$11</definedName>
     <definedName name="Slicer_Representative">#N/A</definedName>
@@ -32,10 +32,10 @@
   <pivotCaches>
     <pivotCache cacheId="0" r:id="rId6"/>
     <pivotCache cacheId="1" r:id="rId7"/>
-    <pivotCache cacheId="9" r:id="rId8"/>
-    <pivotCache cacheId="12" r:id="rId9"/>
-    <pivotCache cacheId="15" r:id="rId10"/>
-    <pivotCache cacheId="18" r:id="rId11"/>
+    <pivotCache cacheId="69" r:id="rId8"/>
+    <pivotCache cacheId="72" r:id="rId9"/>
+    <pivotCache cacheId="75" r:id="rId10"/>
+    <pivotCache cacheId="78" r:id="rId11"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{876F7934-8845-4945-9796-88D515C7AA90}">
@@ -111,7 +111,7 @@
     <extLst>
       <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{DE250136-89BD-433C-8126-D09CA5730AF9}">
         <x15:connection id="calls" autoDelete="1">
-          <x15:rangePr sourceName="_xlcn.WorksheetConnection_excel_portfolioproject.xlsxcalls"/>
+          <x15:rangePr sourceName="_xlcn.WorksheetConnection_excel_portfolioproject.xlsxcalls1"/>
         </x15:connection>
       </ext>
     </extLst>
@@ -120,7 +120,7 @@
     <extLst>
       <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{DE250136-89BD-433C-8126-D09CA5730AF9}">
         <x15:connection id="customers">
-          <x15:rangePr sourceName="_xlcn.WorksheetConnection_excel_portfolioproject.xlsxcustomers"/>
+          <x15:rangePr sourceName="_xlcn.WorksheetConnection_excel_portfolioproject.xlsxcustomers1"/>
         </x15:connection>
       </ext>
     </extLst>
@@ -4128,13 +4128,13 @@
                   <c:v>#N/A</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>207</c:v>
+                  <c:v>#N/A</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>#N/A</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>#N/A</c:v>
+                  <c:v>200</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -4566,13 +4566,13 @@
                   <c:v>#N/A</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>20872</c:v>
+                  <c:v>#N/A</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>#N/A</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>#N/A</c:v>
+                  <c:v>20104</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -5059,25 +5059,25 @@
                 <c:formatCode>#,##0</c:formatCode>
                 <c:ptCount val="7"/>
                 <c:pt idx="0">
-                  <c:v>30</c:v>
+                  <c:v>27</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>34</c:v>
+                  <c:v>22</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>26</c:v>
+                  <c:v>27</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>38</c:v>
+                  <c:v>27</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>27</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>27</c:v>
+                  <c:v>32</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>25</c:v>
+                  <c:v>38</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -5691,40 +5691,40 @@
                 <c:formatCode>#,##0</c:formatCode>
                 <c:ptCount val="12"/>
                 <c:pt idx="0">
-                  <c:v>13</c:v>
+                  <c:v>21</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>13</c:v>
+                  <c:v>18</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>28</c:v>
+                  <c:v>31</c:v>
                 </c:pt>
                 <c:pt idx="3">
+                  <c:v>20</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>8</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>12</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>12</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>7</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>20</c:v>
+                </c:pt>
+                <c:pt idx="9">
                   <c:v>24</c:v>
                 </c:pt>
-                <c:pt idx="4">
-                  <c:v>23</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>17</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>11</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>11</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>14</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>30</c:v>
-                </c:pt>
                 <c:pt idx="10">
-                  <c:v>14</c:v>
+                  <c:v>12</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>9</c:v>
+                  <c:v>15</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -5848,40 +5848,40 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="12"/>
                 <c:pt idx="0">
-                  <c:v>13</c:v>
+                  <c:v>21</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>13</c:v>
+                  <c:v>18</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>28</c:v>
+                  <c:v>31</c:v>
                 </c:pt>
                 <c:pt idx="3">
+                  <c:v>20</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>8</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>12</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>12</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>7</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>20</c:v>
+                </c:pt>
+                <c:pt idx="9">
                   <c:v>24</c:v>
                 </c:pt>
-                <c:pt idx="4">
-                  <c:v>23</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>17</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>11</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>11</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>14</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>30</c:v>
-                </c:pt>
                 <c:pt idx="10">
-                  <c:v>14</c:v>
+                  <c:v>12</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>9</c:v>
+                  <c:v>15</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -6384,13 +6384,13 @@
                   <c:v>#N/A</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>20872</c:v>
+                  <c:v>#N/A</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>#N/A</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>#N/A</c:v>
+                  <c:v>20104</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -6841,13 +6841,13 @@
                   <c:v>#N/A</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>207</c:v>
+                  <c:v>#N/A</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>#N/A</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>#N/A</c:v>
+                  <c:v>200</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -10664,7 +10664,7 @@
               <a:cs typeface="Times New Roman"/>
             </a:rPr>
             <a:pPr algn="ctr"/>
-            <a:t>207</a:t>
+            <a:t>200</a:t>
           </a:fld>
           <a:endParaRPr lang="en-IN" sz="1100">
             <a:solidFill>
@@ -10960,7 +10960,7 @@
               <a:cs typeface="Times New Roman"/>
             </a:rPr>
             <a:pPr marL="0" indent="0" algn="ctr"/>
-            <a:t>₹ 20,872</a:t>
+            <a:t>₹ 20,104</a:t>
           </a:fld>
           <a:endParaRPr lang="en-IN" sz="1100" b="0" i="0" u="none" strike="noStrike">
             <a:solidFill>
@@ -11205,7 +11205,7 @@
               <a:cs typeface="Times New Roman"/>
             </a:rPr>
             <a:pPr marL="0" indent="0" algn="ctr"/>
-            <a:t>17700</a:t>
+            <a:t>18209</a:t>
           </a:fld>
           <a:endParaRPr lang="en-IN" sz="1100" b="0" i="0" u="none" strike="noStrike">
             <a:solidFill>
@@ -11724,7 +11724,7 @@
               <a:cs typeface="Times New Roman"/>
             </a:rPr>
             <a:pPr marL="0" indent="0" algn="ctr"/>
-            <a:t>60</a:t>
+            <a:t>51</a:t>
           </a:fld>
           <a:endParaRPr lang="en-IN" sz="1200" b="0" i="0" u="none" strike="noStrike">
             <a:solidFill>
@@ -11891,18 +11891,18 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>15</xdr:col>
-      <xdr:colOff>221510</xdr:colOff>
+      <xdr:colOff>8859</xdr:colOff>
       <xdr:row>16</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:rowOff>26582</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>301255</xdr:colOff>
-      <xdr:row>25</xdr:row>
-      <xdr:rowOff>8860</xdr:rowOff>
+      <xdr:colOff>354418</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>168349</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
-      <mc:Choice Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
         <xdr:graphicFrame macro="">
           <xdr:nvGraphicFramePr>
             <xdr:cNvPr id="37" name="Representative 1">
@@ -11925,7 +11925,7 @@
           </a:graphic>
         </xdr:graphicFrame>
       </mc:Choice>
-      <mc:Fallback xmlns="">
+      <mc:Fallback>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="0" name=""/>
@@ -11935,8 +11935,8 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="8594650" y="2835349"/>
-              <a:ext cx="1302489" cy="1603744"/>
+              <a:off x="8381999" y="2861931"/>
+              <a:ext cx="1568303" cy="1559441"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
               <a:avLst/>
@@ -13072,7 +13072,7 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition3.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" saveData="0" refreshedBy="sivanagajyothi yedururu" refreshedDate="45756.574839814813" backgroundQuery="1" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="0" supportSubquery="1" supportAdvancedDrill="1" xr:uid="{75F358FF-AB0D-499A-93F7-81A3139FEAE8}">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" saveData="0" refreshedBy="sivanagajyothi yedururu" refreshedDate="45756.576075578705" backgroundQuery="1" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="0" supportSubquery="1" supportAdvancedDrill="1" xr:uid="{75F358FF-AB0D-499A-93F7-81A3139FEAE8}">
   <cacheSource type="external" connectionId="2"/>
   <cacheFields count="6">
     <cacheField name="[Measures].[call count]" caption="call count" numFmtId="0" hierarchy="17" level="32767"/>
@@ -13167,7 +13167,7 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition4.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" saveData="0" refreshedBy="sivanagajyothi yedururu" refreshedDate="45756.574840972222" backgroundQuery="1" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="0" supportSubquery="1" supportAdvancedDrill="1" xr:uid="{5159991F-E602-45B4-B5A0-E05043722C99}">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" saveData="0" refreshedBy="sivanagajyothi yedururu" refreshedDate="45756.576076273152" backgroundQuery="1" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="0" supportSubquery="1" supportAdvancedDrill="1" xr:uid="{5159991F-E602-45B4-B5A0-E05043722C99}">
   <cacheSource type="external" connectionId="2"/>
   <cacheFields count="5">
     <cacheField name="[calls].[Representative].[Representative]" caption="Representative" numFmtId="0" hierarchy="3" level="1">
@@ -13434,7 +13434,7 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition5.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" saveData="0" refreshedBy="sivanagajyothi yedururu" refreshedDate="45756.574842013892" backgroundQuery="1" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="0" supportSubquery="1" supportAdvancedDrill="1" xr:uid="{B3312215-48F3-48DA-84C7-101967613022}">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" saveData="0" refreshedBy="sivanagajyothi yedururu" refreshedDate="45756.576076620368" backgroundQuery="1" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="0" supportSubquery="1" supportAdvancedDrill="1" xr:uid="{B3312215-48F3-48DA-84C7-101967613022}">
   <cacheSource type="external" connectionId="2"/>
   <cacheFields count="3">
     <cacheField name="[calls].[Representative].[Representative]" caption="Representative" numFmtId="0" hierarchy="3" level="1">
@@ -13525,12 +13525,12 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition6.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" saveData="0" refreshedBy="sivanagajyothi yedururu" refreshedDate="45756.574842708331" backgroundQuery="1" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="0" supportSubquery="1" supportAdvancedDrill="1" xr:uid="{92373610-BC8A-4D70-A8C7-01427099730D}">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" saveData="0" refreshedBy="sivanagajyothi yedururu" refreshedDate="45756.576077199075" backgroundQuery="1" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="0" supportSubquery="1" supportAdvancedDrill="1" xr:uid="{92373610-BC8A-4D70-A8C7-01427099730D}">
   <cacheSource type="external" connectionId="2"/>
   <cacheFields count="1">
     <cacheField name="[calls].[Representative].[Representative]" caption="Representative" numFmtId="0" hierarchy="3" level="1">
       <sharedItems count="1">
-        <s v="R03"/>
+        <s v="R05"/>
       </sharedItems>
     </cacheField>
   </cacheFields>
@@ -13643,7 +13643,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{AAB53815-8D20-4469-8EC4-4352A86443FA}" name="weekly trend" cacheId="15" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" subtotalHiddenItems="1" itemPrintTitles="1" createdVersion="8" indent="0" multipleFieldFilters="0" chartFormat="23">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{AAB53815-8D20-4469-8EC4-4352A86443FA}" name="weekly trend" cacheId="75" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" subtotalHiddenItems="1" itemPrintTitles="1" createdVersion="8" indent="0" multipleFieldFilters="0" chartFormat="23">
   <location ref="E19:F27" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="3">
     <pivotField allDrilled="1" showAll="0" dataSourceSort="1" defaultAttributeDrillState="1"/>
@@ -13731,7 +13731,7 @@
     <pivotHierarchy dragToData="1"/>
     <pivotHierarchy multipleItemSelectionAllowed="1" dragToData="1">
       <members count="1" level="1">
-        <member name="[calls].[Representative].&amp;[R03]"/>
+        <member name="[calls].[Representative].&amp;[R05]"/>
       </members>
     </pivotHierarchy>
     <pivotHierarchy dragToData="1"/>
@@ -13778,7 +13778,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{0CE4B034-F5D3-48CB-8B96-4EDB0797DC50}" name="month trend" cacheId="12" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" subtotalHiddenItems="1" itemPrintTitles="1" createdVersion="8" indent="0" multipleFieldFilters="0" chartFormat="11">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{0CE4B034-F5D3-48CB-8B96-4EDB0797DC50}" name="month trend" cacheId="72" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" subtotalHiddenItems="1" itemPrintTitles="1" createdVersion="8" indent="0" multipleFieldFilters="0" chartFormat="11">
   <location ref="A19:C32" firstHeaderRow="0" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="5">
     <pivotField allDrilled="1" showAll="0" dataSourceSort="1" defaultAttributeDrillState="1"/>
@@ -14051,7 +14051,7 @@
     <pivotHierarchy dragToData="1"/>
     <pivotHierarchy multipleItemSelectionAllowed="1" dragToData="1">
       <members count="1" level="1">
-        <member name="[calls].[Representative].&amp;[R03]"/>
+        <member name="[calls].[Representative].&amp;[R05]"/>
       </members>
     </pivotHierarchy>
     <pivotHierarchy dragToData="1"/>
@@ -14102,7 +14102,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{2C89DBDB-5792-4DE1-B0D8-F6BE6B3A85F2}" name="rep pivot" cacheId="9" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" subtotalHiddenItems="1" itemPrintTitles="1" createdVersion="8" indent="0" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{2C89DBDB-5792-4DE1-B0D8-F6BE6B3A85F2}" name="rep pivot" cacheId="69" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" subtotalHiddenItems="1" itemPrintTitles="1" createdVersion="8" indent="0" multipleFieldFilters="0">
   <location ref="A11:E12" firstHeaderRow="0" firstDataRow="1" firstDataCol="0"/>
   <pivotFields count="6">
     <pivotField dataField="1" showAll="0"/>
@@ -14148,7 +14148,7 @@
     <pivotHierarchy dragToData="1"/>
     <pivotHierarchy multipleItemSelectionAllowed="1" dragToData="1">
       <members count="1" level="1">
-        <member name="[calls].[Representative].&amp;[R03]"/>
+        <member name="[calls].[Representative].&amp;[R05]"/>
       </members>
     </pivotHierarchy>
     <pivotHierarchy dragToData="1"/>
@@ -14283,7 +14283,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable5.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{D9FABC9E-27C8-4580-ADE9-CEF021B283CD}" name="selected_rep_pivot" cacheId="18" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{D9FABC9E-27C8-4580-ADE9-CEF021B283CD}" name="selected_rep_pivot" cacheId="78" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" multipleFieldFilters="0">
   <location ref="A58:A60" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="1">
     <pivotField axis="axisRow" allDrilled="1" showAll="0" dataSourceSort="1" defaultAttributeDrillState="1">
@@ -14527,7 +14527,7 @@
         </level>
       </levels>
       <selections count="1">
-        <selection n="[calls].[Representative].&amp;[R03]"/>
+        <selection n="[calls].[Representative].&amp;[R05]"/>
       </selections>
     </olap>
   </data>
@@ -14542,7 +14542,7 @@
 
 <file path=xl/slicers/slicer2.xml><?xml version="1.0" encoding="utf-8"?>
 <slicers xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x xr10">
-  <slicer name="Representative 1" xr10:uid="{8841FB45-53E1-4D33-91C1-E6CBC71CFBF8}" cache="Slicer_Representative" caption="Representative" level="1" rowHeight="222250"/>
+  <slicer name="Representative 1" xr10:uid="{8841FB45-53E1-4D33-91C1-E6CBC71CFBF8}" cache="Slicer_Representative" caption="Representative" level="1" style="SlicerStyleOther2" rowHeight="222250"/>
 </slicers>
 </file>
 
@@ -22520,8 +22520,9 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
   <tableParts count="1">
-    <tablePart r:id="rId1"/>
+    <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
 </file>
@@ -22593,19 +22594,19 @@
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="21">
-        <v>207</v>
+        <v>200</v>
       </c>
       <c r="B12" s="30">
-        <v>20872</v>
+        <v>20104</v>
       </c>
       <c r="C12" s="23">
-        <v>17700</v>
+        <v>18209</v>
       </c>
       <c r="D12" s="23">
-        <v>3.9275362318840581</v>
+        <v>3.9350000000000001</v>
       </c>
       <c r="E12" s="23">
-        <v>60</v>
+        <v>51</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
@@ -22630,16 +22631,16 @@
         <v>1073</v>
       </c>
       <c r="B20" s="31">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="C20" s="21">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="E20" s="27" t="s">
         <v>1058</v>
       </c>
       <c r="F20" s="21">
-        <v>30</v>
+        <v>27</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
@@ -22647,16 +22648,16 @@
         <v>1074</v>
       </c>
       <c r="B21" s="31">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="C21" s="21">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="E21" s="27" t="s">
         <v>1066</v>
       </c>
       <c r="F21" s="21">
-        <v>34</v>
+        <v>22</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
@@ -22664,16 +22665,16 @@
         <v>1075</v>
       </c>
       <c r="B22" s="31">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="C22" s="21">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="E22" s="27" t="s">
         <v>1060</v>
       </c>
       <c r="F22" s="21">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
@@ -22681,16 +22682,16 @@
         <v>1076</v>
       </c>
       <c r="B23" s="31">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="C23" s="21">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="E23" s="27" t="s">
         <v>1062</v>
       </c>
       <c r="F23" s="21">
-        <v>38</v>
+        <v>27</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.25">
@@ -22698,10 +22699,10 @@
         <v>1077</v>
       </c>
       <c r="B24" s="31">
-        <v>23</v>
+        <v>8</v>
       </c>
       <c r="C24" s="21">
-        <v>23</v>
+        <v>8</v>
       </c>
       <c r="E24" s="27" t="s">
         <v>1064</v>
@@ -22715,16 +22716,16 @@
         <v>1078</v>
       </c>
       <c r="B25" s="31">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="C25" s="21">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="E25" s="27" t="s">
         <v>1067</v>
       </c>
       <c r="F25" s="21">
-        <v>27</v>
+        <v>32</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.25">
@@ -22732,16 +22733,16 @@
         <v>1079</v>
       </c>
       <c r="B26" s="31">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C26" s="21">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E26" s="27" t="s">
         <v>1065</v>
       </c>
       <c r="F26" s="21">
-        <v>25</v>
+        <v>38</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.25">
@@ -22749,16 +22750,16 @@
         <v>1080</v>
       </c>
       <c r="B27" s="31">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="C27" s="21">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="E27" s="27" t="s">
         <v>1072</v>
       </c>
       <c r="F27" s="21">
-        <v>207</v>
+        <v>200</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
@@ -22766,10 +22767,10 @@
         <v>1081</v>
       </c>
       <c r="B28" s="31">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="C28" s="21">
-        <v>14</v>
+        <v>20</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.25">
@@ -22777,10 +22778,10 @@
         <v>1082</v>
       </c>
       <c r="B29" s="31">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="C29" s="21">
-        <v>30</v>
+        <v>24</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.25">
@@ -22788,10 +22789,10 @@
         <v>1083</v>
       </c>
       <c r="B30" s="31">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="C30" s="21">
-        <v>14</v>
+        <v>12</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.25">
@@ -22799,10 +22800,10 @@
         <v>1084</v>
       </c>
       <c r="B31" s="31">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="C31" s="21">
-        <v>9</v>
+        <v>15</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.25">
@@ -22810,10 +22811,10 @@
         <v>1072</v>
       </c>
       <c r="B32" s="31">
-        <v>207</v>
+        <v>200</v>
       </c>
       <c r="C32" s="21">
-        <v>207</v>
+        <v>200</v>
       </c>
     </row>
     <row r="40" spans="1:9" x14ac:dyDescent="0.25">
@@ -22822,7 +22823,7 @@
       </c>
       <c r="G40" t="str">
         <f>A59</f>
-        <v>R03</v>
+        <v>R05</v>
       </c>
       <c r="H40" t="s">
         <v>1091</v>
@@ -22831,7 +22832,7 @@
     <row r="41" spans="1:9" x14ac:dyDescent="0.25">
       <c r="H41" t="str">
         <f>A59</f>
-        <v>R03</v>
+        <v>R05</v>
       </c>
     </row>
     <row r="42" spans="1:9" x14ac:dyDescent="0.25">
@@ -22927,13 +22928,13 @@
       <c r="G45" s="29">
         <v>20872</v>
       </c>
-      <c r="H45">
+      <c r="H45" t="e">
         <f t="shared" si="0"/>
-        <v>207</v>
-      </c>
-      <c r="I45" s="29">
+        <v>#N/A</v>
+      </c>
+      <c r="I45" s="29" t="e">
         <f t="shared" si="1"/>
-        <v>20872</v>
+        <v>#N/A</v>
       </c>
     </row>
     <row r="46" spans="1:9" x14ac:dyDescent="0.25">
@@ -22983,13 +22984,13 @@
       <c r="G47" s="29">
         <v>20104</v>
       </c>
-      <c r="H47" t="e">
+      <c r="H47">
         <f t="shared" si="0"/>
-        <v>#N/A</v>
-      </c>
-      <c r="I47" s="29" t="e">
+        <v>200</v>
+      </c>
+      <c r="I47" s="29">
         <f t="shared" si="1"/>
-        <v>#N/A</v>
+        <v>20104</v>
       </c>
     </row>
     <row r="48" spans="1:9" x14ac:dyDescent="0.25">
@@ -23021,7 +23022,7 @@
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A59" s="28" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
     </row>
     <row r="60" spans="1:3" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Commentless GitLatch Commit @ 2025-4-9-13-57-29-102
</commit_message>
<xml_diff>
--- a/excel_portfolioproject.xlsx
+++ b/excel_portfolioproject.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yedur\OneDrive\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F7264FCA-5584-451A-995B-8834A4525ECC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{0808BAAE-FEFB-4006-9AB7-7258888816F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{26D4546B-D2A1-4444-8EAF-A6228F96F0C1}"/>
   </bookViews>
@@ -32,10 +32,10 @@
   <pivotCaches>
     <pivotCache cacheId="0" r:id="rId6"/>
     <pivotCache cacheId="1" r:id="rId7"/>
-    <pivotCache cacheId="69" r:id="rId8"/>
-    <pivotCache cacheId="72" r:id="rId9"/>
-    <pivotCache cacheId="75" r:id="rId10"/>
-    <pivotCache cacheId="78" r:id="rId11"/>
+    <pivotCache cacheId="129" r:id="rId8"/>
+    <pivotCache cacheId="132" r:id="rId9"/>
+    <pivotCache cacheId="135" r:id="rId10"/>
+    <pivotCache cacheId="138" r:id="rId11"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{876F7934-8845-4945-9796-88D515C7AA90}">
@@ -10439,6 +10439,84 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>8860</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>26582</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>17</xdr:col>
+      <xdr:colOff>141768</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>168349</xdr:rowOff>
+    </xdr:to>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+        <xdr:graphicFrame macro="">
+          <xdr:nvGraphicFramePr>
+            <xdr:cNvPr id="37" name="Representative 1">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{22315FB6-DE9E-40B0-A336-746FD371B032}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvGraphicFramePr/>
+          </xdr:nvGraphicFramePr>
+          <xdr:xfrm>
+            <a:off x="0" y="0"/>
+            <a:ext cx="0" cy="0"/>
+          </xdr:xfrm>
+          <a:graphic>
+            <a:graphicData uri="http://schemas.microsoft.com/office/drawing/2010/slicer">
+              <sle:slicer xmlns:sle="http://schemas.microsoft.com/office/drawing/2010/slicer" name="Representative 1"/>
+            </a:graphicData>
+          </a:graphic>
+        </xdr:graphicFrame>
+      </mc:Choice>
+      <mc:Fallback>
+        <xdr:sp macro="" textlink="">
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="0" name=""/>
+            <xdr:cNvSpPr>
+              <a:spLocks noTextEdit="1"/>
+            </xdr:cNvSpPr>
+          </xdr:nvSpPr>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="8382000" y="2861931"/>
+              <a:ext cx="1355652" cy="1559441"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:solidFill>
+              <a:prstClr val="white"/>
+            </a:solidFill>
+            <a:ln w="1">
+              <a:solidFill>
+                <a:prstClr val="green"/>
+              </a:solidFill>
+            </a:ln>
+          </xdr:spPr>
+          <xdr:txBody>
+            <a:bodyPr vertOverflow="clip" horzOverflow="clip"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:r>
+                <a:rPr lang="en-IN" sz="1100"/>
+                <a:t>This shape represents a slicer. Slicers are supported in Excel 2010 or later.
+If the shape was modified in an earlier version of Excel, or if the workbook was saved in Excel 2003 or earlier, the slicer cannot be used.</a:t>
+              </a:r>
+            </a:p>
+          </xdr:txBody>
+        </xdr:sp>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>182880</xdr:colOff>
       <xdr:row>2</xdr:row>
@@ -11888,84 +11966,6 @@
     </xdr:pic>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>15</xdr:col>
-      <xdr:colOff>8859</xdr:colOff>
-      <xdr:row>16</xdr:row>
-      <xdr:rowOff>26582</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>17</xdr:col>
-      <xdr:colOff>354418</xdr:colOff>
-      <xdr:row>24</xdr:row>
-      <xdr:rowOff>168349</xdr:rowOff>
-    </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
-        <xdr:graphicFrame macro="">
-          <xdr:nvGraphicFramePr>
-            <xdr:cNvPr id="37" name="Representative 1">
-              <a:extLst>
-                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{22315FB6-DE9E-40B0-A336-746FD371B032}"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPr>
-            <xdr:cNvGraphicFramePr/>
-          </xdr:nvGraphicFramePr>
-          <xdr:xfrm>
-            <a:off x="0" y="0"/>
-            <a:ext cx="0" cy="0"/>
-          </xdr:xfrm>
-          <a:graphic>
-            <a:graphicData uri="http://schemas.microsoft.com/office/drawing/2010/slicer">
-              <sle:slicer xmlns:sle="http://schemas.microsoft.com/office/drawing/2010/slicer" name="Representative 1"/>
-            </a:graphicData>
-          </a:graphic>
-        </xdr:graphicFrame>
-      </mc:Choice>
-      <mc:Fallback>
-        <xdr:sp macro="" textlink="">
-          <xdr:nvSpPr>
-            <xdr:cNvPr id="0" name=""/>
-            <xdr:cNvSpPr>
-              <a:spLocks noTextEdit="1"/>
-            </xdr:cNvSpPr>
-          </xdr:nvSpPr>
-          <xdr:spPr>
-            <a:xfrm>
-              <a:off x="8381999" y="2861931"/>
-              <a:ext cx="1568303" cy="1559441"/>
-            </a:xfrm>
-            <a:prstGeom prst="rect">
-              <a:avLst/>
-            </a:prstGeom>
-            <a:solidFill>
-              <a:prstClr val="white"/>
-            </a:solidFill>
-            <a:ln w="1">
-              <a:solidFill>
-                <a:prstClr val="green"/>
-              </a:solidFill>
-            </a:ln>
-          </xdr:spPr>
-          <xdr:txBody>
-            <a:bodyPr vertOverflow="clip" horzOverflow="clip"/>
-            <a:lstStyle/>
-            <a:p>
-              <a:r>
-                <a:rPr lang="en-IN" sz="1100"/>
-                <a:t>This shape represents a slicer. Slicers are supported in Excel 2010 or later.
-If the shape was modified in an earlier version of Excel, or if the workbook was saved in Excel 2003 or earlier, the slicer cannot be used.</a:t>
-              </a:r>
-            </a:p>
-          </xdr:txBody>
-        </xdr:sp>
-      </mc:Fallback>
-    </mc:AlternateContent>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>11</xdr:col>
@@ -13072,7 +13072,7 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition3.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" saveData="0" refreshedBy="sivanagajyothi yedururu" refreshedDate="45756.576075578705" backgroundQuery="1" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="0" supportSubquery="1" supportAdvancedDrill="1" xr:uid="{75F358FF-AB0D-499A-93F7-81A3139FEAE8}">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" saveData="0" refreshedBy="sivanagajyothi yedururu" refreshedDate="45756.577913078705" backgroundQuery="1" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="0" supportSubquery="1" supportAdvancedDrill="1" xr:uid="{75F358FF-AB0D-499A-93F7-81A3139FEAE8}">
   <cacheSource type="external" connectionId="2"/>
   <cacheFields count="6">
     <cacheField name="[Measures].[call count]" caption="call count" numFmtId="0" hierarchy="17" level="32767"/>
@@ -13167,7 +13167,7 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition4.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" saveData="0" refreshedBy="sivanagajyothi yedururu" refreshedDate="45756.576076273152" backgroundQuery="1" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="0" supportSubquery="1" supportAdvancedDrill="1" xr:uid="{5159991F-E602-45B4-B5A0-E05043722C99}">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" saveData="0" refreshedBy="sivanagajyothi yedururu" refreshedDate="45756.577913657406" backgroundQuery="1" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="0" supportSubquery="1" supportAdvancedDrill="1" xr:uid="{5159991F-E602-45B4-B5A0-E05043722C99}">
   <cacheSource type="external" connectionId="2"/>
   <cacheFields count="5">
     <cacheField name="[calls].[Representative].[Representative]" caption="Representative" numFmtId="0" hierarchy="3" level="1">
@@ -13434,7 +13434,7 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition5.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" saveData="0" refreshedBy="sivanagajyothi yedururu" refreshedDate="45756.576076620368" backgroundQuery="1" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="0" supportSubquery="1" supportAdvancedDrill="1" xr:uid="{B3312215-48F3-48DA-84C7-101967613022}">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" saveData="0" refreshedBy="sivanagajyothi yedururu" refreshedDate="45756.577914120367" backgroundQuery="1" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="0" supportSubquery="1" supportAdvancedDrill="1" xr:uid="{B3312215-48F3-48DA-84C7-101967613022}">
   <cacheSource type="external" connectionId="2"/>
   <cacheFields count="3">
     <cacheField name="[calls].[Representative].[Representative]" caption="Representative" numFmtId="0" hierarchy="3" level="1">
@@ -13525,7 +13525,7 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition6.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" saveData="0" refreshedBy="sivanagajyothi yedururu" refreshedDate="45756.576077199075" backgroundQuery="1" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="0" supportSubquery="1" supportAdvancedDrill="1" xr:uid="{92373610-BC8A-4D70-A8C7-01427099730D}">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" saveData="0" refreshedBy="sivanagajyothi yedururu" refreshedDate="45756.577914467591" backgroundQuery="1" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="0" supportSubquery="1" supportAdvancedDrill="1" xr:uid="{92373610-BC8A-4D70-A8C7-01427099730D}">
   <cacheSource type="external" connectionId="2"/>
   <cacheFields count="1">
     <cacheField name="[calls].[Representative].[Representative]" caption="Representative" numFmtId="0" hierarchy="3" level="1">
@@ -13643,7 +13643,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{AAB53815-8D20-4469-8EC4-4352A86443FA}" name="weekly trend" cacheId="75" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" subtotalHiddenItems="1" itemPrintTitles="1" createdVersion="8" indent="0" multipleFieldFilters="0" chartFormat="23">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{AAB53815-8D20-4469-8EC4-4352A86443FA}" name="weekly trend" cacheId="135" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" subtotalHiddenItems="1" itemPrintTitles="1" createdVersion="8" indent="0" multipleFieldFilters="0" chartFormat="23">
   <location ref="E19:F27" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="3">
     <pivotField allDrilled="1" showAll="0" dataSourceSort="1" defaultAttributeDrillState="1"/>
@@ -13778,7 +13778,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{0CE4B034-F5D3-48CB-8B96-4EDB0797DC50}" name="month trend" cacheId="72" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" subtotalHiddenItems="1" itemPrintTitles="1" createdVersion="8" indent="0" multipleFieldFilters="0" chartFormat="11">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{0CE4B034-F5D3-48CB-8B96-4EDB0797DC50}" name="month trend" cacheId="132" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" subtotalHiddenItems="1" itemPrintTitles="1" createdVersion="8" indent="0" multipleFieldFilters="0" chartFormat="11">
   <location ref="A19:C32" firstHeaderRow="0" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="5">
     <pivotField allDrilled="1" showAll="0" dataSourceSort="1" defaultAttributeDrillState="1"/>
@@ -14102,7 +14102,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{2C89DBDB-5792-4DE1-B0D8-F6BE6B3A85F2}" name="rep pivot" cacheId="69" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" subtotalHiddenItems="1" itemPrintTitles="1" createdVersion="8" indent="0" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{2C89DBDB-5792-4DE1-B0D8-F6BE6B3A85F2}" name="rep pivot" cacheId="129" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" subtotalHiddenItems="1" itemPrintTitles="1" createdVersion="8" indent="0" multipleFieldFilters="0">
   <location ref="A11:E12" firstHeaderRow="0" firstDataRow="1" firstDataCol="0"/>
   <pivotFields count="6">
     <pivotField dataField="1" showAll="0"/>
@@ -14283,7 +14283,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable5.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{D9FABC9E-27C8-4580-ADE9-CEF021B283CD}" name="selected_rep_pivot" cacheId="78" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{D9FABC9E-27C8-4580-ADE9-CEF021B283CD}" name="selected_rep_pivot" cacheId="138" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" multipleFieldFilters="0">
   <location ref="A58:A60" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="1">
     <pivotField axis="axisRow" allDrilled="1" showAll="0" dataSourceSort="1" defaultAttributeDrillState="1">
@@ -14542,7 +14542,7 @@
 
 <file path=xl/slicers/slicer2.xml><?xml version="1.0" encoding="utf-8"?>
 <slicers xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x xr10">
-  <slicer name="Representative 1" xr10:uid="{8841FB45-53E1-4D33-91C1-E6CBC71CFBF8}" cache="Slicer_Representative" caption="Representative" level="1" style="SlicerStyleOther2" rowHeight="222250"/>
+  <slicer name="Representative 1" xr10:uid="{8841FB45-53E1-4D33-91C1-E6CBC71CFBF8}" cache="Slicer_Representative" caption="Representative" level="1" style="SlicerStyleDark5" rowHeight="222250"/>
 </slicers>
 </file>
 
@@ -14810,7 +14810,7 @@
 
 <file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
 <wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
-  <wetp:taskpane dockstate="right" visibility="1" width="438" row="6">
+  <wetp:taskpane dockstate="right" visibility="1" width="438" row="7">
     <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </wetp:taskpane>
 </wetp:taskpanes>

</xml_diff>

<commit_message>
Commentless GitLatch Commit @ 2025-4-9-19-33-6-636
</commit_message>
<xml_diff>
--- a/excel_portfolioproject.xlsx
+++ b/excel_portfolioproject.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yedur\OneDrive\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{0808BAAE-FEFB-4006-9AB7-7258888816F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{7D3A4B21-EC89-4E3B-A3E3-DF925E5247D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{26D4546B-D2A1-4444-8EAF-A6228F96F0C1}"/>
   </bookViews>
@@ -30,22 +30,23 @@
   </definedNames>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="0" r:id="rId6"/>
-    <pivotCache cacheId="1" r:id="rId7"/>
-    <pivotCache cacheId="129" r:id="rId8"/>
-    <pivotCache cacheId="132" r:id="rId9"/>
-    <pivotCache cacheId="135" r:id="rId10"/>
-    <pivotCache cacheId="138" r:id="rId11"/>
+    <pivotCache cacheId="19" r:id="rId6"/>
+    <pivotCache cacheId="20" r:id="rId7"/>
+    <pivotCache cacheId="21" r:id="rId8"/>
+    <pivotCache cacheId="22" r:id="rId9"/>
+    <pivotCache cacheId="23" r:id="rId10"/>
+    <pivotCache cacheId="24" r:id="rId11"/>
+    <pivotCache cacheId="33" r:id="rId12"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{876F7934-8845-4945-9796-88D515C7AA90}">
       <x14:pivotCaches>
-        <pivotCache cacheId="6" r:id="rId12"/>
+        <pivotCache cacheId="6" r:id="rId13"/>
       </x14:pivotCaches>
     </ext>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{BBE1A952-AA13-448e-AADC-164F8A28A991}">
       <x14:slicerCaches>
-        <x14:slicerCache r:id="rId13"/>
+        <x14:slicerCache r:id="rId14"/>
       </x14:slicerCaches>
     </ext>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{79F54976-1DA5-4618-B147-4CDE4B953A38}">
@@ -151,7 +152,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4225" uniqueCount="1093">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4235" uniqueCount="1094">
   <si>
     <t>Customer ID</t>
   </si>
@@ -3430,17 +3431,19 @@
   </si>
   <si>
     <t>sel amount</t>
+  </si>
+  <si>
+    <t>Column Labels</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
-  <numFmts count="4">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="[$-409]d\-mmm\-yy;@"/>
     <numFmt numFmtId="165" formatCode="&quot;₹&quot;\ #,##0;#,##0\ \-&quot;₹&quot;;&quot;₹&quot;\ #,##0"/>
     <numFmt numFmtId="166" formatCode="&quot;₹&quot;\ #,##0"/>
-    <numFmt numFmtId="167" formatCode="&quot;₹&quot;\ #,##0;#,##0\ \-&quot;₹&quot;;&quot;₹&quot;\ #,##0"/>
   </numFmts>
   <fonts count="4" x14ac:knownFonts="1">
     <font>
@@ -3620,7 +3623,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
@@ -3667,8 +3670,6 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3865,871 +3866,6 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
-  <c:date1904 val="0"/>
-  <c:lang val="en-US"/>
-  <c:roundedCorners val="0"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
-      <c14:style val="102"/>
-    </mc:Choice>
-    <mc:Fallback>
-      <c:style val="2"/>
-    </mc:Fallback>
-  </mc:AlternateContent>
-  <c:chart>
-    <c:title>
-      <c:overlay val="0"/>
-      <c:spPr>
-        <a:noFill/>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-        <a:effectLst/>
-      </c:spPr>
-      <c:txPr>
-        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr>
-            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
-              <a:solidFill>
-                <a:schemeClr val="tx1">
-                  <a:lumMod val="65000"/>
-                  <a:lumOff val="35000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:defRPr>
-          </a:pPr>
-          <a:endParaRPr lang="en-US"/>
-        </a:p>
-      </c:txPr>
-    </c:title>
-    <c:autoTitleDeleted val="0"/>
-    <c:plotArea>
-      <c:layout/>
-      <c:barChart>
-        <c:barDir val="bar"/>
-        <c:grouping val="clustered"/>
-        <c:varyColors val="0"/>
-        <c:ser>
-          <c:idx val="0"/>
-          <c:order val="0"/>
-          <c:spPr>
-            <a:solidFill>
-              <a:schemeClr val="bg1">
-                <a:lumMod val="65000"/>
-              </a:schemeClr>
-            </a:solidFill>
-            <a:ln>
-              <a:noFill/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:invertIfNegative val="0"/>
-          <c:dLbls>
-            <c:spPr>
-              <a:noFill/>
-              <a:ln>
-                <a:noFill/>
-              </a:ln>
-              <a:effectLst/>
-            </c:spPr>
-            <c:txPr>
-              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
-                <a:spAutoFit/>
-              </a:bodyPr>
-              <a:lstStyle/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                    <a:solidFill>
-                      <a:schemeClr val="tx1">
-                        <a:lumMod val="75000"/>
-                        <a:lumOff val="25000"/>
-                      </a:schemeClr>
-                    </a:solidFill>
-                    <a:latin typeface="+mn-lt"/>
-                    <a:ea typeface="+mn-ea"/>
-                    <a:cs typeface="+mn-cs"/>
-                  </a:defRPr>
-                </a:pPr>
-                <a:endParaRPr lang="en-US"/>
-              </a:p>
-            </c:txPr>
-            <c:dLblPos val="outEnd"/>
-            <c:showLegendKey val="0"/>
-            <c:showVal val="1"/>
-            <c:showCatName val="0"/>
-            <c:showSerName val="0"/>
-            <c:showPercent val="0"/>
-            <c:showBubbleSize val="0"/>
-            <c:showLeaderLines val="0"/>
-            <c:extLst>
-              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
-                <c15:showLeaderLines val="1"/>
-                <c15:leaderLines>
-                  <c:spPr>
-                    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-                      <a:solidFill>
-                        <a:schemeClr val="tx1">
-                          <a:lumMod val="35000"/>
-                          <a:lumOff val="65000"/>
-                        </a:schemeClr>
-                      </a:solidFill>
-                      <a:round/>
-                    </a:ln>
-                    <a:effectLst/>
-                  </c:spPr>
-                </c15:leaderLines>
-              </c:ext>
-            </c:extLst>
-          </c:dLbls>
-          <c:cat>
-            <c:strRef>
-              <c:f>pivot!$E$43:$E$47</c:f>
-              <c:strCache>
-                <c:ptCount val="5"/>
-                <c:pt idx="0">
-                  <c:v>R01</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>R02</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>R03</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>R04</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>R05</c:v>
-                </c:pt>
-              </c:strCache>
-            </c:strRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>pivot!$F$43:$F$47</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="5"/>
-                <c:pt idx="0">
-                  <c:v>189</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>218</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>207</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>186</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>200</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:val>
-          <c:extLst>
-            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-57C2-4550-9A7E-A16A6D5EDB8C}"/>
-            </c:ext>
-          </c:extLst>
-        </c:ser>
-        <c:ser>
-          <c:idx val="1"/>
-          <c:order val="1"/>
-          <c:tx>
-            <c:v>sel.calls</c:v>
-          </c:tx>
-          <c:spPr>
-            <a:solidFill>
-              <a:srgbClr val="FF0000"/>
-            </a:solidFill>
-            <a:ln>
-              <a:noFill/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:invertIfNegative val="0"/>
-          <c:dLbls>
-            <c:spPr>
-              <a:noFill/>
-              <a:ln>
-                <a:noFill/>
-              </a:ln>
-              <a:effectLst/>
-            </c:spPr>
-            <c:txPr>
-              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
-                <a:spAutoFit/>
-              </a:bodyPr>
-              <a:lstStyle/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                    <a:solidFill>
-                      <a:schemeClr val="tx1">
-                        <a:lumMod val="75000"/>
-                        <a:lumOff val="25000"/>
-                      </a:schemeClr>
-                    </a:solidFill>
-                    <a:latin typeface="+mn-lt"/>
-                    <a:ea typeface="+mn-ea"/>
-                    <a:cs typeface="+mn-cs"/>
-                  </a:defRPr>
-                </a:pPr>
-                <a:endParaRPr lang="en-US"/>
-              </a:p>
-            </c:txPr>
-            <c:dLblPos val="outEnd"/>
-            <c:showLegendKey val="0"/>
-            <c:showVal val="1"/>
-            <c:showCatName val="0"/>
-            <c:showSerName val="0"/>
-            <c:showPercent val="0"/>
-            <c:showBubbleSize val="0"/>
-            <c:showLeaderLines val="0"/>
-            <c:extLst>
-              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
-                <c15:showLeaderLines val="1"/>
-                <c15:leaderLines>
-                  <c:spPr>
-                    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-                      <a:solidFill>
-                        <a:schemeClr val="tx1">
-                          <a:lumMod val="35000"/>
-                          <a:lumOff val="65000"/>
-                        </a:schemeClr>
-                      </a:solidFill>
-                      <a:round/>
-                    </a:ln>
-                    <a:effectLst/>
-                  </c:spPr>
-                </c15:leaderLines>
-              </c:ext>
-            </c:extLst>
-          </c:dLbls>
-          <c:val>
-            <c:numRef>
-              <c:f>pivot!$H$43:$H$47</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="5"/>
-                <c:pt idx="0">
-                  <c:v>#N/A</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>#N/A</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>#N/A</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>#N/A</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>200</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:val>
-          <c:extLst>
-            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-57C2-4550-9A7E-A16A6D5EDB8C}"/>
-            </c:ext>
-          </c:extLst>
-        </c:ser>
-        <c:dLbls>
-          <c:dLblPos val="outEnd"/>
-          <c:showLegendKey val="0"/>
-          <c:showVal val="1"/>
-          <c:showCatName val="0"/>
-          <c:showSerName val="0"/>
-          <c:showPercent val="0"/>
-          <c:showBubbleSize val="0"/>
-        </c:dLbls>
-        <c:gapWidth val="25"/>
-        <c:overlap val="100"/>
-        <c:axId val="1439431727"/>
-        <c:axId val="1439432207"/>
-      </c:barChart>
-      <c:catAx>
-        <c:axId val="1439431727"/>
-        <c:scaling>
-          <c:orientation val="maxMin"/>
-        </c:scaling>
-        <c:delete val="0"/>
-        <c:axPos val="l"/>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
-        <c:majorTickMark val="out"/>
-        <c:minorTickMark val="none"/>
-        <c:tickLblPos val="nextTo"/>
-        <c:spPr>
-          <a:noFill/>
-          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-            <a:solidFill>
-              <a:schemeClr val="tx1">
-                <a:lumMod val="15000"/>
-                <a:lumOff val="85000"/>
-              </a:schemeClr>
-            </a:solidFill>
-            <a:round/>
-          </a:ln>
-          <a:effectLst/>
-        </c:spPr>
-        <c:txPr>
-          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                <a:solidFill>
-                  <a:schemeClr val="tx1">
-                    <a:lumMod val="65000"/>
-                    <a:lumOff val="35000"/>
-                  </a:schemeClr>
-                </a:solidFill>
-                <a:latin typeface="+mn-lt"/>
-                <a:ea typeface="+mn-ea"/>
-                <a:cs typeface="+mn-cs"/>
-              </a:defRPr>
-            </a:pPr>
-            <a:endParaRPr lang="en-US"/>
-          </a:p>
-        </c:txPr>
-        <c:crossAx val="1439432207"/>
-        <c:crosses val="autoZero"/>
-        <c:auto val="1"/>
-        <c:lblAlgn val="ctr"/>
-        <c:lblOffset val="100"/>
-        <c:noMultiLvlLbl val="0"/>
-      </c:catAx>
-      <c:valAx>
-        <c:axId val="1439432207"/>
-        <c:scaling>
-          <c:orientation val="minMax"/>
-        </c:scaling>
-        <c:delete val="1"/>
-        <c:axPos val="t"/>
-        <c:majorGridlines>
-          <c:spPr>
-            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-              <a:solidFill>
-                <a:schemeClr val="tx1">
-                  <a:lumMod val="15000"/>
-                  <a:lumOff val="85000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-        </c:majorGridlines>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
-        <c:majorTickMark val="out"/>
-        <c:minorTickMark val="none"/>
-        <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="1439431727"/>
-        <c:crosses val="autoZero"/>
-        <c:crossBetween val="between"/>
-      </c:valAx>
-      <c:spPr>
-        <a:noFill/>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-        <a:effectLst/>
-      </c:spPr>
-    </c:plotArea>
-    <c:plotVisOnly val="1"/>
-    <c:dispBlanksAs val="gap"/>
-    <c:extLst>
-      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
-        <c16r3:dataDisplayOptions16>
-          <c16r3:dispNaAsBlank val="1"/>
-        </c16r3:dataDisplayOptions16>
-      </c:ext>
-    </c:extLst>
-    <c:showDLblsOverMax val="0"/>
-  </c:chart>
-  <c:spPr>
-    <a:solidFill>
-      <a:schemeClr val="bg1"/>
-    </a:solidFill>
-    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-      <a:solidFill>
-        <a:schemeClr val="tx1">
-          <a:lumMod val="15000"/>
-          <a:lumOff val="85000"/>
-        </a:schemeClr>
-      </a:solidFill>
-      <a:round/>
-    </a:ln>
-    <a:effectLst/>
-  </c:spPr>
-  <c:txPr>
-    <a:bodyPr/>
-    <a:lstStyle/>
-    <a:p>
-      <a:pPr>
-        <a:defRPr/>
-      </a:pPr>
-      <a:endParaRPr lang="en-US"/>
-    </a:p>
-  </c:txPr>
-  <c:printSettings>
-    <c:headerFooter/>
-    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
-    <c:pageSetup/>
-  </c:printSettings>
-</c:chartSpace>
-</file>
-
-<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
-  <c:date1904 val="0"/>
-  <c:lang val="en-US"/>
-  <c:roundedCorners val="0"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
-      <c14:style val="102"/>
-    </mc:Choice>
-    <mc:Fallback>
-      <c:style val="2"/>
-    </mc:Fallback>
-  </mc:AlternateContent>
-  <c:clrMapOvr bg1="lt1" tx1="dk1" bg2="lt2" tx2="dk2" accent1="accent1" accent2="accent2" accent3="accent3" accent4="accent4" accent5="accent5" accent6="accent6" hlink="hlink" folHlink="folHlink"/>
-  <c:chart>
-    <c:title>
-      <c:overlay val="0"/>
-      <c:spPr>
-        <a:noFill/>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-        <a:effectLst/>
-      </c:spPr>
-      <c:txPr>
-        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr>
-            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
-              <a:solidFill>
-                <a:schemeClr val="tx1">
-                  <a:lumMod val="65000"/>
-                  <a:lumOff val="35000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:defRPr>
-          </a:pPr>
-          <a:endParaRPr lang="en-US"/>
-        </a:p>
-      </c:txPr>
-    </c:title>
-    <c:autoTitleDeleted val="0"/>
-    <c:plotArea>
-      <c:layout>
-        <c:manualLayout>
-          <c:layoutTarget val="inner"/>
-          <c:xMode val="edge"/>
-          <c:yMode val="edge"/>
-          <c:x val="0.12025863692875713"/>
-          <c:y val="0.15787037037037038"/>
-          <c:w val="0.83986895477778201"/>
-          <c:h val="0.78194444444444444"/>
-        </c:manualLayout>
-      </c:layout>
-      <c:barChart>
-        <c:barDir val="bar"/>
-        <c:grouping val="clustered"/>
-        <c:varyColors val="0"/>
-        <c:ser>
-          <c:idx val="0"/>
-          <c:order val="0"/>
-          <c:spPr>
-            <a:solidFill>
-              <a:sysClr val="window" lastClr="FFFFFF">
-                <a:lumMod val="65000"/>
-              </a:sysClr>
-            </a:solidFill>
-            <a:ln>
-              <a:noFill/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:invertIfNegative val="0"/>
-          <c:dLbls>
-            <c:spPr>
-              <a:noFill/>
-              <a:ln>
-                <a:noFill/>
-              </a:ln>
-              <a:effectLst/>
-            </c:spPr>
-            <c:txPr>
-              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
-                <a:spAutoFit/>
-              </a:bodyPr>
-              <a:lstStyle/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                    <a:solidFill>
-                      <a:schemeClr val="tx1">
-                        <a:lumMod val="75000"/>
-                        <a:lumOff val="25000"/>
-                      </a:schemeClr>
-                    </a:solidFill>
-                    <a:latin typeface="+mn-lt"/>
-                    <a:ea typeface="+mn-ea"/>
-                    <a:cs typeface="+mn-cs"/>
-                  </a:defRPr>
-                </a:pPr>
-                <a:endParaRPr lang="en-US"/>
-              </a:p>
-            </c:txPr>
-            <c:dLblPos val="outEnd"/>
-            <c:showLegendKey val="0"/>
-            <c:showVal val="1"/>
-            <c:showCatName val="0"/>
-            <c:showSerName val="0"/>
-            <c:showPercent val="0"/>
-            <c:showBubbleSize val="0"/>
-            <c:showLeaderLines val="0"/>
-            <c:extLst>
-              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
-                <c15:showLeaderLines val="1"/>
-                <c15:leaderLines>
-                  <c:spPr>
-                    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-                      <a:solidFill>
-                        <a:schemeClr val="tx1">
-                          <a:lumMod val="35000"/>
-                          <a:lumOff val="65000"/>
-                        </a:schemeClr>
-                      </a:solidFill>
-                      <a:round/>
-                    </a:ln>
-                    <a:effectLst/>
-                  </c:spPr>
-                </c15:leaderLines>
-              </c:ext>
-            </c:extLst>
-          </c:dLbls>
-          <c:cat>
-            <c:strRef>
-              <c:f>pivot!$E$43:$E$47</c:f>
-              <c:strCache>
-                <c:ptCount val="5"/>
-                <c:pt idx="0">
-                  <c:v>R01</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>R02</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>R03</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>R04</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>R05</c:v>
-                </c:pt>
-              </c:strCache>
-            </c:strRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>pivot!$G$43:$G$47</c:f>
-              <c:numCache>
-                <c:formatCode>"₹"\ #,##0</c:formatCode>
-                <c:ptCount val="5"/>
-                <c:pt idx="0">
-                  <c:v>18415</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>20581</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>20872</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>16651</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>20104</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:val>
-          <c:extLst>
-            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-BA21-4D9C-828A-E1F7D73DDC40}"/>
-            </c:ext>
-          </c:extLst>
-        </c:ser>
-        <c:ser>
-          <c:idx val="1"/>
-          <c:order val="1"/>
-          <c:tx>
-            <c:v>sel.amount</c:v>
-          </c:tx>
-          <c:spPr>
-            <a:solidFill>
-              <a:srgbClr val="F14124"/>
-            </a:solidFill>
-            <a:ln>
-              <a:noFill/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:invertIfNegative val="0"/>
-          <c:dLbls>
-            <c:spPr>
-              <a:noFill/>
-              <a:ln>
-                <a:noFill/>
-              </a:ln>
-              <a:effectLst/>
-            </c:spPr>
-            <c:txPr>
-              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
-                <a:spAutoFit/>
-              </a:bodyPr>
-              <a:lstStyle/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                    <a:solidFill>
-                      <a:schemeClr val="tx1">
-                        <a:lumMod val="75000"/>
-                        <a:lumOff val="25000"/>
-                      </a:schemeClr>
-                    </a:solidFill>
-                    <a:latin typeface="+mn-lt"/>
-                    <a:ea typeface="+mn-ea"/>
-                    <a:cs typeface="+mn-cs"/>
-                  </a:defRPr>
-                </a:pPr>
-                <a:endParaRPr lang="en-US"/>
-              </a:p>
-            </c:txPr>
-            <c:dLblPos val="outEnd"/>
-            <c:showLegendKey val="0"/>
-            <c:showVal val="1"/>
-            <c:showCatName val="0"/>
-            <c:showSerName val="0"/>
-            <c:showPercent val="0"/>
-            <c:showBubbleSize val="0"/>
-            <c:showLeaderLines val="0"/>
-            <c:extLst>
-              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
-                <c15:showLeaderLines val="1"/>
-                <c15:leaderLines>
-                  <c:spPr>
-                    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-                      <a:solidFill>
-                        <a:schemeClr val="tx1">
-                          <a:lumMod val="35000"/>
-                          <a:lumOff val="65000"/>
-                        </a:schemeClr>
-                      </a:solidFill>
-                      <a:round/>
-                    </a:ln>
-                    <a:effectLst/>
-                  </c:spPr>
-                </c15:leaderLines>
-              </c:ext>
-            </c:extLst>
-          </c:dLbls>
-          <c:val>
-            <c:numRef>
-              <c:f>pivot!$I$43:$I$48</c:f>
-              <c:numCache>
-                <c:formatCode>"₹"\ #,##0</c:formatCode>
-                <c:ptCount val="6"/>
-                <c:pt idx="0">
-                  <c:v>#N/A</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>#N/A</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>#N/A</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>#N/A</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>20104</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:val>
-          <c:extLst>
-            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{0000000B-BA21-4D9C-828A-E1F7D73DDC40}"/>
-            </c:ext>
-          </c:extLst>
-        </c:ser>
-        <c:dLbls>
-          <c:dLblPos val="outEnd"/>
-          <c:showLegendKey val="0"/>
-          <c:showVal val="1"/>
-          <c:showCatName val="0"/>
-          <c:showSerName val="0"/>
-          <c:showPercent val="0"/>
-          <c:showBubbleSize val="0"/>
-        </c:dLbls>
-        <c:gapWidth val="25"/>
-        <c:overlap val="100"/>
-        <c:axId val="1439431727"/>
-        <c:axId val="1439432207"/>
-      </c:barChart>
-      <c:catAx>
-        <c:axId val="1439431727"/>
-        <c:scaling>
-          <c:orientation val="maxMin"/>
-        </c:scaling>
-        <c:delete val="0"/>
-        <c:axPos val="l"/>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
-        <c:majorTickMark val="out"/>
-        <c:minorTickMark val="none"/>
-        <c:tickLblPos val="nextTo"/>
-        <c:spPr>
-          <a:noFill/>
-          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-            <a:solidFill>
-              <a:schemeClr val="tx1">
-                <a:lumMod val="15000"/>
-                <a:lumOff val="85000"/>
-              </a:schemeClr>
-            </a:solidFill>
-            <a:round/>
-          </a:ln>
-          <a:effectLst/>
-        </c:spPr>
-        <c:txPr>
-          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                <a:solidFill>
-                  <a:schemeClr val="tx1">
-                    <a:lumMod val="65000"/>
-                    <a:lumOff val="35000"/>
-                  </a:schemeClr>
-                </a:solidFill>
-                <a:latin typeface="+mn-lt"/>
-                <a:ea typeface="+mn-ea"/>
-                <a:cs typeface="+mn-cs"/>
-              </a:defRPr>
-            </a:pPr>
-            <a:endParaRPr lang="en-US"/>
-          </a:p>
-        </c:txPr>
-        <c:crossAx val="1439432207"/>
-        <c:crosses val="autoZero"/>
-        <c:auto val="1"/>
-        <c:lblAlgn val="ctr"/>
-        <c:lblOffset val="100"/>
-        <c:noMultiLvlLbl val="0"/>
-      </c:catAx>
-      <c:valAx>
-        <c:axId val="1439432207"/>
-        <c:scaling>
-          <c:orientation val="minMax"/>
-        </c:scaling>
-        <c:delete val="1"/>
-        <c:axPos val="t"/>
-        <c:majorGridlines>
-          <c:spPr>
-            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-              <a:solidFill>
-                <a:schemeClr val="tx1">
-                  <a:lumMod val="15000"/>
-                  <a:lumOff val="85000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-        </c:majorGridlines>
-        <c:numFmt formatCode="&quot;₹&quot;\ #,##0" sourceLinked="1"/>
-        <c:majorTickMark val="out"/>
-        <c:minorTickMark val="none"/>
-        <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="1439431727"/>
-        <c:crosses val="autoZero"/>
-        <c:crossBetween val="between"/>
-      </c:valAx>
-      <c:spPr>
-        <a:noFill/>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-        <a:effectLst/>
-      </c:spPr>
-    </c:plotArea>
-    <c:plotVisOnly val="1"/>
-    <c:dispBlanksAs val="gap"/>
-    <c:extLst>
-      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
-        <c16r3:dataDisplayOptions16>
-          <c16r3:dispNaAsBlank val="1"/>
-        </c16r3:dataDisplayOptions16>
-      </c:ext>
-    </c:extLst>
-    <c:showDLblsOverMax val="0"/>
-  </c:chart>
-  <c:spPr>
-    <a:solidFill>
-      <a:schemeClr val="bg1"/>
-    </a:solidFill>
-    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-      <a:solidFill>
-        <a:schemeClr val="tx1">
-          <a:lumMod val="15000"/>
-          <a:lumOff val="85000"/>
-        </a:schemeClr>
-      </a:solidFill>
-      <a:round/>
-    </a:ln>
-    <a:effectLst/>
-  </c:spPr>
-  <c:txPr>
-    <a:bodyPr/>
-    <a:lstStyle/>
-    <a:p>
-      <a:pPr>
-        <a:defRPr/>
-      </a:pPr>
-      <a:endParaRPr lang="en-US"/>
-    </a:p>
-  </c:txPr>
-  <c:printSettings>
-    <c:headerFooter/>
-    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
-    <c:pageSetup/>
-  </c:printSettings>
-</c:chartSpace>
-</file>
-
-<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
   <c:lang val="en-US"/>
@@ -5259,7 +4395,7 @@
 </c:chartSpace>
 </file>
 
-<file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
   <c:lang val="en-US"/>
@@ -6080,7 +5216,7 @@
 </c:chartSpace>
 </file>
 
-<file path=xl/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
   <c:lang val="en-US"/>
@@ -6540,7 +5676,7 @@
 </c:chartSpace>
 </file>
 
-<file path=xl/charts/chart6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
   <c:lang val="en-US"/>
@@ -6997,6 +6133,781 @@
 </c:chartSpace>
 </file>
 
+<file path=xl/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:pivotSource>
+    <c:name>[excel_portfolioproject.xlsx]pivot!PivotTable1</c:name>
+    <c:fmtId val="3"/>
+  </c:pivotSource>
+  <c:chart>
+    <c:autoTitleDeleted val="0"/>
+    <c:pivotFmts>
+      <c:pivotFmt>
+        <c:idx val="0"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:marker>
+          <c:symbol val="none"/>
+        </c:marker>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="1"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:marker>
+          <c:symbol val="none"/>
+        </c:marker>
+        <c:dLbl>
+          <c:idx val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:spAutoFit/>
+            </a:bodyPr>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="75000"/>
+                      <a:lumOff val="25000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+          </c:extLst>
+        </c:dLbl>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="2"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:marker>
+          <c:symbol val="none"/>
+        </c:marker>
+        <c:dLbl>
+          <c:idx val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:spAutoFit/>
+            </a:bodyPr>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="75000"/>
+                      <a:lumOff val="25000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+          </c:extLst>
+        </c:dLbl>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="3"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:marker>
+          <c:symbol val="none"/>
+        </c:marker>
+        <c:dLbl>
+          <c:idx val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:spAutoFit/>
+            </a:bodyPr>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="75000"/>
+                      <a:lumOff val="25000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+          </c:extLst>
+        </c:dLbl>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="4"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent5"/>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:marker>
+          <c:symbol val="none"/>
+        </c:marker>
+        <c:dLbl>
+          <c:idx val="0"/>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="lt1"/>
+            </a:solidFill>
+            <a:ln>
+              <a:solidFill>
+                <a:schemeClr val="dk1">
+                  <a:lumMod val="25000"/>
+                  <a:lumOff val="75000"/>
+                </a:schemeClr>
+              </a:solidFill>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+              <a:spAutoFit/>
+            </a:bodyPr>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="dk1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+          <c:dLblPos val="ctr"/>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="1"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+              <c15:spPr xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
+                <a:prstGeom prst="roundRect">
+                  <a:avLst/>
+                </a:prstGeom>
+                <a:noFill/>
+                <a:ln>
+                  <a:noFill/>
+                </a:ln>
+              </c15:spPr>
+            </c:ext>
+          </c:extLst>
+        </c:dLbl>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="5"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent4"/>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:marker>
+          <c:symbol val="none"/>
+        </c:marker>
+        <c:dLbl>
+          <c:idx val="0"/>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="lt1"/>
+            </a:solidFill>
+            <a:ln>
+              <a:solidFill>
+                <a:schemeClr val="dk1">
+                  <a:lumMod val="25000"/>
+                  <a:lumOff val="75000"/>
+                </a:schemeClr>
+              </a:solidFill>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+              <a:spAutoFit/>
+            </a:bodyPr>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="dk1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+          <c:dLblPos val="ctr"/>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="1"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+              <c15:spPr xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
+                <a:prstGeom prst="roundRect">
+                  <a:avLst/>
+                </a:prstGeom>
+                <a:noFill/>
+                <a:ln>
+                  <a:noFill/>
+                </a:ln>
+              </c15:spPr>
+            </c:ext>
+          </c:extLst>
+        </c:dLbl>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="6"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent5"/>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+      </c:pivotFmt>
+    </c:pivotFmts>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="percentStacked"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>pivot!$E$55:$E$56</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Female</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent5"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:dLbls>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:ln>
+                <a:solidFill>
+                  <a:schemeClr val="dk1">
+                    <a:lumMod val="25000"/>
+                    <a:lumOff val="75000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:txPr>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+                <a:spAutoFit/>
+              </a:bodyPr>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="dk1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="en-US"/>
+              </a:p>
+            </c:txPr>
+            <c:dLblPos val="ctr"/>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="1"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:showBubbleSize val="0"/>
+            <c:showLeaderLines val="0"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:spPr xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
+                  <a:prstGeom prst="roundRect">
+                    <a:avLst/>
+                  </a:prstGeom>
+                  <a:noFill/>
+                  <a:ln>
+                    <a:noFill/>
+                  </a:ln>
+                </c15:spPr>
+                <c15:showLeaderLines val="1"/>
+                <c15:leaderLines>
+                  <c:spPr>
+                    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+                      <a:solidFill>
+                        <a:schemeClr val="tx1">
+                          <a:lumMod val="35000"/>
+                          <a:lumOff val="65000"/>
+                        </a:schemeClr>
+                      </a:solidFill>
+                      <a:round/>
+                    </a:ln>
+                    <a:effectLst/>
+                  </c:spPr>
+                </c15:leaderLines>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>pivot!$D$57:$D$60</c:f>
+              <c:strCache>
+                <c:ptCount val="3"/>
+                <c:pt idx="0">
+                  <c:v>Cincinnati</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Cleveland</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Columbus</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>pivot!$E$57:$E$60</c:f>
+              <c:numCache>
+                <c:formatCode>#,##0</c:formatCode>
+                <c:ptCount val="3"/>
+                <c:pt idx="0">
+                  <c:v>144</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>326</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>129</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-CBB7-43E0-A250-1399056AC033}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>pivot!$F$55:$F$56</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Male</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent4"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:dLbls>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:ln>
+                <a:solidFill>
+                  <a:schemeClr val="dk1">
+                    <a:lumMod val="25000"/>
+                    <a:lumOff val="75000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:txPr>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+                <a:spAutoFit/>
+              </a:bodyPr>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="dk1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="en-US"/>
+              </a:p>
+            </c:txPr>
+            <c:dLblPos val="ctr"/>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="1"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:showBubbleSize val="0"/>
+            <c:showLeaderLines val="0"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:spPr xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
+                  <a:prstGeom prst="roundRect">
+                    <a:avLst/>
+                  </a:prstGeom>
+                  <a:noFill/>
+                  <a:ln>
+                    <a:noFill/>
+                  </a:ln>
+                </c15:spPr>
+                <c15:showLeaderLines val="1"/>
+                <c15:leaderLines>
+                  <c:spPr>
+                    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+                      <a:solidFill>
+                        <a:schemeClr val="tx1">
+                          <a:lumMod val="35000"/>
+                          <a:lumOff val="65000"/>
+                        </a:schemeClr>
+                      </a:solidFill>
+                      <a:round/>
+                    </a:ln>
+                    <a:effectLst/>
+                  </c:spPr>
+                </c15:leaderLines>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>pivot!$D$57:$D$60</c:f>
+              <c:strCache>
+                <c:ptCount val="3"/>
+                <c:pt idx="0">
+                  <c:v>Cincinnati</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Cleveland</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Columbus</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>pivot!$F$57:$F$60</c:f>
+              <c:numCache>
+                <c:formatCode>#,##0</c:formatCode>
+                <c:ptCount val="3"/>
+                <c:pt idx="0">
+                  <c:v>132</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>63</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>206</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-CBB7-43E0-A250-1399056AC033}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:gapWidth val="25"/>
+        <c:overlap val="100"/>
+        <c:axId val="1169520496"/>
+        <c:axId val="1169515216"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="1169520496"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="1"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="1169515216"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="1169515216"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="1"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="0%" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="1169520496"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+  <c:userShapes r:id="rId3"/>
+  <c:extLst>
+    <c:ext xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" uri="{781A3756-C4B2-4CAC-9D66-4F8BD8637D16}">
+      <c14:pivotOptions>
+        <c14:dropZoneFilter val="1"/>
+        <c14:dropZoneCategories val="1"/>
+        <c14:dropZoneData val="1"/>
+      </c14:pivotOptions>
+    </c:ext>
+    <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{E28EC0CA-F0BB-4C9C-879D-F8772B89E7AC}">
+      <c16:pivotOptions16>
+        <c16:showExpandCollapseFieldButtons val="1"/>
+      </c16:pivotOptions16>
+    </c:ext>
+  </c:extLst>
+</c:chartSpace>
+</file>
+
 <file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
   <a:schemeClr val="accent1"/>
@@ -7158,46 +7069,6 @@
 </file>
 
 <file path=xl/charts/colors5.xml><?xml version="1.0" encoding="utf-8"?>
-<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
-  <a:schemeClr val="accent1"/>
-  <a:schemeClr val="accent2"/>
-  <a:schemeClr val="accent3"/>
-  <a:schemeClr val="accent4"/>
-  <a:schemeClr val="accent5"/>
-  <a:schemeClr val="accent6"/>
-  <cs:variation/>
-  <cs:variation>
-    <a:lumMod val="60000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="80000"/>
-    <a:lumOff val="20000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="80000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="60000"/>
-    <a:lumOff val="40000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="50000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="70000"/>
-    <a:lumOff val="30000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="70000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="50000"/>
-    <a:lumOff val="50000"/>
-  </cs:variation>
-</cs:colorStyle>
-</file>
-
-<file path=xl/charts/colors6.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
   <a:schemeClr val="accent1"/>
   <a:schemeClr val="accent2"/>
@@ -7743,7 +7614,7 @@
 </file>
 
 <file path=xl/charts/style2.xml><?xml version="1.0" encoding="utf-8"?>
-<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="216">
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="322">
   <cs:axisTitle>
     <cs:lnRef idx="0"/>
     <cs:fillRef idx="0"/>
@@ -8068,8 +7939,8 @@
       <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
         <a:solidFill>
           <a:schemeClr val="tx1">
-            <a:lumMod val="50000"/>
-            <a:lumOff val="50000"/>
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
           </a:schemeClr>
         </a:solidFill>
         <a:round/>
@@ -8133,6 +8004,17 @@
         <a:lumOff val="35000"/>
       </a:schemeClr>
     </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
     <cs:defRPr sz="900" kern="1200"/>
   </cs:seriesAxis>
   <cs:seriesLine>
@@ -8753,522 +8635,6 @@
 </file>
 
 <file path=xl/charts/style4.xml><?xml version="1.0" encoding="utf-8"?>
-<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="322">
-  <cs:axisTitle>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="1000" kern="1200"/>
-  </cs:axisTitle>
-  <cs:categoryAxis>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:categoryAxis>
-  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="bg1"/>
-      </a:solidFill>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="1000" kern="1200"/>
-  </cs:chartArea>
-  <cs:dataLabel>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="75000"/>
-        <a:lumOff val="25000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:dataLabel>
-  <cs:dataLabelCallout>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="lt1"/>
-      </a:solidFill>
-      <a:ln>
-        <a:solidFill>
-          <a:schemeClr val="dk1">
-            <a:lumMod val="25000"/>
-            <a:lumOff val="75000"/>
-          </a:schemeClr>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
-    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
-      <a:spAutoFit/>
-    </cs:bodyPr>
-  </cs:dataLabelCallout>
-  <cs:dataPoint>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="1">
-      <cs:styleClr val="auto"/>
-    </cs:fillRef>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-  </cs:dataPoint>
-  <cs:dataPoint3D>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="1">
-      <cs:styleClr val="auto"/>
-    </cs:fillRef>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-  </cs:dataPoint3D>
-  <cs:dataPointLine>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="1"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="28575" cap="rnd">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:dataPointLine>
-  <cs:dataPointMarker>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="1">
-      <cs:styleClr val="auto"/>
-    </cs:fillRef>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-  </cs:dataPointMarker>
-  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
-  <cs:dataPointWireframe>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="1"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="rnd">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:dataPointWireframe>
-  <cs:dataTable>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:noFill/>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:dataTable>
-  <cs:downBar>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="dk1">
-          <a:lumMod val="75000"/>
-          <a:lumOff val="25000"/>
-        </a:schemeClr>
-      </a:solidFill>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="65000"/>
-            <a:lumOff val="35000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:downBar>
-  <cs:dropLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="35000"/>
-            <a:lumOff val="65000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:dropLine>
-  <cs:errorBar>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="65000"/>
-            <a:lumOff val="35000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:errorBar>
-  <cs:floor>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:noFill/>
-      <a:ln>
-        <a:noFill/>
-      </a:ln>
-    </cs:spPr>
-  </cs:floor>
-  <cs:gridlineMajor>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:gridlineMajor>
-  <cs:gridlineMinor>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="5000"/>
-            <a:lumOff val="95000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:gridlineMinor>
-  <cs:hiLoLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="75000"/>
-            <a:lumOff val="25000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:hiLoLine>
-  <cs:leaderLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="35000"/>
-            <a:lumOff val="65000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:leaderLine>
-  <cs:legend>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:legend>
-  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-  </cs:plotArea>
-  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-  </cs:plotArea3D>
-  <cs:seriesAxis>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:seriesAxis>
-  <cs:seriesLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="35000"/>
-            <a:lumOff val="65000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:seriesLine>
-  <cs:title>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
-  </cs:title>
-  <cs:trendline>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="19050" cap="rnd">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:prstDash val="sysDot"/>
-      </a:ln>
-    </cs:spPr>
-  </cs:trendline>
-  <cs:trendlineLabel>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:trendlineLabel>
-  <cs:upBar>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="lt1"/>
-      </a:solidFill>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="65000"/>
-            <a:lumOff val="35000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:upBar>
-  <cs:valueAxis>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:valueAxis>
-  <cs:wall>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:noFill/>
-      <a:ln>
-        <a:noFill/>
-      </a:ln>
-    </cs:spPr>
-  </cs:wall>
-</cs:chartStyle>
-</file>
-
-<file path=xl/charts/style5.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="216">
   <cs:axisTitle>
     <cs:lnRef idx="0"/>
@@ -9773,8 +9139,8 @@
 </cs:chartStyle>
 </file>
 
-<file path=xl/charts/style6.xml><?xml version="1.0" encoding="utf-8"?>
-<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="216">
+<file path=xl/charts/style5.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="297">
   <cs:axisTitle>
     <cs:lnRef idx="0"/>
     <cs:fillRef idx="0"/>
@@ -10358,80 +9724,6 @@
     </mc:AlternateContent>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>11</xdr:col>
-      <xdr:colOff>441960</xdr:colOff>
-      <xdr:row>47</xdr:row>
-      <xdr:rowOff>137160</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>16</xdr:col>
-      <xdr:colOff>411480</xdr:colOff>
-      <xdr:row>63</xdr:row>
-      <xdr:rowOff>15240</xdr:rowOff>
-    </xdr:to>
-    <xdr:graphicFrame macro="">
-      <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="5" name="Chart 4">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{CA0CD8A3-1182-C6EC-0CE9-595F9CD490FB}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvGraphicFramePr/>
-      </xdr:nvGraphicFramePr>
-      <xdr:xfrm>
-        <a:off x="0" y="0"/>
-        <a:ext cx="0" cy="0"/>
-      </xdr:xfrm>
-      <a:graphic>
-        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-        </a:graphicData>
-      </a:graphic>
-    </xdr:graphicFrame>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>251460</xdr:colOff>
-      <xdr:row>49</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>11</xdr:col>
-      <xdr:colOff>30480</xdr:colOff>
-      <xdr:row>64</xdr:row>
-      <xdr:rowOff>114300</xdr:rowOff>
-    </xdr:to>
-    <xdr:graphicFrame macro="">
-      <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="6" name="Chart 5">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{06299A88-B486-438D-AF8E-725D0125EAF4}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvGraphicFramePr>
-          <a:graphicFrameLocks/>
-        </xdr:cNvGraphicFramePr>
-      </xdr:nvGraphicFramePr>
-      <xdr:xfrm>
-        <a:off x="0" y="0"/>
-        <a:ext cx="0" cy="0"/>
-      </xdr:xfrm>
-      <a:graphic>
-        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
-        </a:graphicData>
-      </a:graphic>
-    </xdr:graphicFrame>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -10450,8 +9742,8 @@
       <xdr:row>24</xdr:row>
       <xdr:rowOff>168349</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
         <xdr:graphicFrame macro="">
           <xdr:nvGraphicFramePr>
             <xdr:cNvPr id="37" name="Representative 1">
@@ -10474,7 +9766,7 @@
           </a:graphic>
         </xdr:graphicFrame>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="0" name=""/>
@@ -12181,10 +11473,293 @@
     </xdr:graphicFrame>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>17</xdr:col>
+      <xdr:colOff>44302</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>26582</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>21</xdr:col>
+      <xdr:colOff>407581</xdr:colOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>44301</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="3" name="Chart 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{0893B3AB-2099-4C0D-85C2-692771266A49}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr>
+          <a:graphicFrameLocks/>
+        </xdr:cNvGraphicFramePr>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId13"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>20</xdr:col>
+      <xdr:colOff>53163</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>114611</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="567070" cy="239809"/>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="6" name="TextBox 5">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{EB9B4E99-920C-AEE5-9D13-0FD0D1ADD945}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="11483163" y="4899262"/>
+          <a:ext cx="567070" cy="239809"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="accent5">
+            <a:lumMod val="20000"/>
+            <a:lumOff val="80000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="b">
+          <a:spAutoFit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-IN" sz="1000"/>
+            <a:t>female</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>168349</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>44302</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="611371" cy="254493"/>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="22" name="TextBox 21">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{DA6EF4AC-B67A-A2AA-2668-D8EE09563A7B}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="10375605" y="4297325"/>
+          <a:ext cx="611371" cy="254493"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="accent5">
+            <a:lumMod val="20000"/>
+            <a:lumOff val="80000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t">
+          <a:spAutoFit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-IN" sz="1100"/>
+            <a:t>female</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
 </xdr:wsDr>
 </file>
 
 <file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<c:userShapes xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <cdr:relSizeAnchor xmlns:cdr="http://schemas.openxmlformats.org/drawingml/2006/chartDrawing">
+    <cdr:from>
+      <cdr:x>0.41325</cdr:x>
+      <cdr:y>0.62766</cdr:y>
+    </cdr:from>
+    <cdr:to>
+      <cdr:x>0.56782</cdr:x>
+      <cdr:y>0.79433</cdr:y>
+    </cdr:to>
+    <cdr:sp macro="" textlink="">
+      <cdr:nvSpPr>
+        <cdr:cNvPr id="2" name="TextBox 1">
+          <a:extLst xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{FFFDB978-148F-4FB9-8972-35EC16A1716D}"/>
+            </a:ext>
+          </a:extLst>
+        </cdr:cNvPr>
+        <cdr:cNvSpPr txBox="1"/>
+      </cdr:nvSpPr>
+      <cdr:spPr>
+        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:off x="1160721" y="1568302"/>
+          <a:ext cx="434163" cy="416442"/>
+        </a:xfrm>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </cdr:spPr>
+      <cdr:txBody>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" vertOverflow="clip" wrap="none" rtlCol="0"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:endParaRPr lang="en-IN" sz="1100" kern="1200"/>
+        </a:p>
+      </cdr:txBody>
+    </cdr:sp>
+  </cdr:relSizeAnchor>
+  <cdr:relSizeAnchor xmlns:cdr="http://schemas.openxmlformats.org/drawingml/2006/chartDrawing">
+    <cdr:from>
+      <cdr:x>0.50473</cdr:x>
+      <cdr:y>0.60638</cdr:y>
+    </cdr:from>
+    <cdr:to>
+      <cdr:x>0.83028</cdr:x>
+      <cdr:y>0.97234</cdr:y>
+    </cdr:to>
+    <cdr:sp macro="" textlink="">
+      <cdr:nvSpPr>
+        <cdr:cNvPr id="3" name="TextBox 2">
+          <a:extLst xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{BB6009F8-29B6-1664-D7EB-BE799A09A6B3}"/>
+            </a:ext>
+          </a:extLst>
+        </cdr:cNvPr>
+        <cdr:cNvSpPr txBox="1"/>
+      </cdr:nvSpPr>
+      <cdr:spPr>
+        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:off x="1417674" y="1515139"/>
+          <a:ext cx="914400" cy="914400"/>
+        </a:xfrm>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </cdr:spPr>
+      <cdr:txBody>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" vertOverflow="clip" wrap="none" rtlCol="0"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:endParaRPr lang="en-IN" sz="1100" kern="1200"/>
+        </a:p>
+      </cdr:txBody>
+    </cdr:sp>
+  </cdr:relSizeAnchor>
+  <cdr:relSizeAnchor xmlns:cdr="http://schemas.openxmlformats.org/drawingml/2006/chartDrawing">
+    <cdr:from>
+      <cdr:x>0.40379</cdr:x>
+      <cdr:y>0.63404</cdr:y>
+    </cdr:from>
+    <cdr:to>
+      <cdr:x>0.5836</cdr:x>
+      <cdr:y>0.84043</cdr:y>
+    </cdr:to>
+    <cdr:sp macro="" textlink="">
+      <cdr:nvSpPr>
+        <cdr:cNvPr id="4" name="TextBox 3">
+          <a:extLst xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{0FDDE828-1F3C-FC2C-9B7E-853E8BB11E2C}"/>
+            </a:ext>
+          </a:extLst>
+        </cdr:cNvPr>
+        <cdr:cNvSpPr txBox="1"/>
+      </cdr:nvSpPr>
+      <cdr:spPr>
+        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:off x="1134141" y="1584250"/>
+          <a:ext cx="505046" cy="515680"/>
+        </a:xfrm>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </cdr:spPr>
+      <cdr:txBody>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" vertOverflow="clip" wrap="none" rtlCol="0"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:endParaRPr lang="en-IN" sz="1100" kern="1200"/>
+        </a:p>
+      </cdr:txBody>
+    </cdr:sp>
+  </cdr:relSizeAnchor>
+</c:userShapes>
+</file>
+
+<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
@@ -12899,179 +12474,6 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" saveData="0" refreshedBy="sivanagajyothi yedururu" refreshedDate="45755.942241435187" backgroundQuery="1" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="0" supportSubquery="1" supportAdvancedDrill="1" xr:uid="{C9E09126-0EF3-4689-9CCC-21407F27E967}">
-  <cacheSource type="external" connectionId="2"/>
-  <cacheFields count="5">
-    <cacheField name="[Measures].[call count]" caption="call count" numFmtId="0" hierarchy="17" level="32767"/>
-    <cacheField name="[Measures].[total amount]" caption="total amount" numFmtId="0" hierarchy="18" level="32767"/>
-    <cacheField name="[Measures].[total duration]" caption="total duration" numFmtId="0" hierarchy="19" level="32767"/>
-    <cacheField name="[Measures].[avg rating]" caption="avg rating" numFmtId="0" hierarchy="20" level="32767"/>
-    <cacheField name="[Measures].[5*rating]" caption="5*rating" numFmtId="0" hierarchy="21" level="32767"/>
-  </cacheFields>
-  <cacheHierarchies count="26">
-    <cacheHierarchy uniqueName="[calls].[Call number]" caption="Call number" attribute="1" defaultMemberUniqueName="[calls].[Call number].[All]" allUniqueName="[calls].[Call number].[All]" dimensionUniqueName="[calls]" displayFolder="" count="0" memberValueDatatype="130" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[calls].[Customer ID]" caption="Customer ID" attribute="1" defaultMemberUniqueName="[calls].[Customer ID].[All]" allUniqueName="[calls].[Customer ID].[All]" dimensionUniqueName="[calls]" displayFolder="" count="0" memberValueDatatype="130" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[calls].[Duration]" caption="Duration" attribute="1" defaultMemberUniqueName="[calls].[Duration].[All]" allUniqueName="[calls].[Duration].[All]" dimensionUniqueName="[calls]" displayFolder="" count="0" memberValueDatatype="20" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[calls].[Representative]" caption="Representative" attribute="1" defaultMemberUniqueName="[calls].[Representative].[All]" allUniqueName="[calls].[Representative].[All]" dimensionUniqueName="[calls]" displayFolder="" count="0" memberValueDatatype="130" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[calls].[Date of Call]" caption="Date of Call" attribute="1" time="1" defaultMemberUniqueName="[calls].[Date of Call].[All]" allUniqueName="[calls].[Date of Call].[All]" dimensionUniqueName="[calls]" displayFolder="" count="0" memberValueDatatype="7" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[calls].[Purchase Amount]" caption="Purchase Amount" attribute="1" defaultMemberUniqueName="[calls].[Purchase Amount].[All]" allUniqueName="[calls].[Purchase Amount].[All]" dimensionUniqueName="[calls]" displayFolder="" count="0" memberValueDatatype="20" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[calls].[Satisfaction Rating]" caption="Satisfaction Rating" attribute="1" defaultMemberUniqueName="[calls].[Satisfaction Rating].[All]" allUniqueName="[calls].[Satisfaction Rating].[All]" dimensionUniqueName="[calls]" displayFolder="" count="0" memberValueDatatype="5" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[calls].[FY]" caption="FY" attribute="1" defaultMemberUniqueName="[calls].[FY].[All]" allUniqueName="[calls].[FY].[All]" dimensionUniqueName="[calls]" displayFolder="" count="0" memberValueDatatype="20" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[calls].[Day of week]" caption="Day of week" attribute="1" defaultMemberUniqueName="[calls].[Day of week].[All]" allUniqueName="[calls].[Day of week].[All]" dimensionUniqueName="[calls]" displayFolder="" count="0" memberValueDatatype="130" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[calls].[Duration Bucket]" caption="Duration Bucket" attribute="1" defaultMemberUniqueName="[calls].[Duration Bucket].[All]" allUniqueName="[calls].[Duration Bucket].[All]" dimensionUniqueName="[calls]" displayFolder="" count="0" memberValueDatatype="130" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[calls].[Rating rounded]" caption="Rating rounded" attribute="1" defaultMemberUniqueName="[calls].[Rating rounded].[All]" allUniqueName="[calls].[Rating rounded].[All]" dimensionUniqueName="[calls]" displayFolder="" count="0" memberValueDatatype="20" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[calls].[Date of Call (Month)]" caption="Date of Call (Month)" attribute="1" defaultMemberUniqueName="[calls].[Date of Call (Month)].[All]" allUniqueName="[calls].[Date of Call (Month)].[All]" dimensionUniqueName="[calls]" displayFolder="" count="0" memberValueDatatype="130" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[customers].[Customer ID]" caption="Customer ID" attribute="1" defaultMemberUniqueName="[customers].[Customer ID].[All]" allUniqueName="[customers].[Customer ID].[All]" dimensionUniqueName="[customers]" displayFolder="" count="0" memberValueDatatype="130" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[customers].[Gedner]" caption="Gedner" attribute="1" defaultMemberUniqueName="[customers].[Gedner].[All]" allUniqueName="[customers].[Gedner].[All]" dimensionUniqueName="[customers]" displayFolder="" count="0" memberValueDatatype="130" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[customers].[Age]" caption="Age" attribute="1" defaultMemberUniqueName="[customers].[Age].[All]" allUniqueName="[customers].[Age].[All]" dimensionUniqueName="[customers]" displayFolder="" count="0" memberValueDatatype="20" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[customers].[City]" caption="City" attribute="1" defaultMemberUniqueName="[customers].[City].[All]" allUniqueName="[customers].[City].[All]" dimensionUniqueName="[customers]" displayFolder="" count="0" memberValueDatatype="130" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[calls].[Date of Call (Month Index)]" caption="Date of Call (Month Index)" attribute="1" defaultMemberUniqueName="[calls].[Date of Call (Month Index)].[All]" allUniqueName="[calls].[Date of Call (Month Index)].[All]" dimensionUniqueName="[calls]" displayFolder="" count="0" memberValueDatatype="20" unbalanced="0" hidden="1"/>
-    <cacheHierarchy uniqueName="[Measures].[call count]" caption="call count" measure="1" displayFolder="" measureGroup="calls" count="0" oneField="1">
-      <fieldsUsage count="1">
-        <fieldUsage x="0"/>
-      </fieldsUsage>
-    </cacheHierarchy>
-    <cacheHierarchy uniqueName="[Measures].[total amount]" caption="total amount" measure="1" displayFolder="" measureGroup="calls" count="0" oneField="1">
-      <fieldsUsage count="1">
-        <fieldUsage x="1"/>
-      </fieldsUsage>
-    </cacheHierarchy>
-    <cacheHierarchy uniqueName="[Measures].[total duration]" caption="total duration" measure="1" displayFolder="" measureGroup="calls" count="0" oneField="1">
-      <fieldsUsage count="1">
-        <fieldUsage x="2"/>
-      </fieldsUsage>
-    </cacheHierarchy>
-    <cacheHierarchy uniqueName="[Measures].[avg rating]" caption="avg rating" measure="1" displayFolder="" measureGroup="calls" count="0" oneField="1">
-      <fieldsUsage count="1">
-        <fieldUsage x="3"/>
-      </fieldsUsage>
-    </cacheHierarchy>
-    <cacheHierarchy uniqueName="[Measures].[5*rating]" caption="5*rating" measure="1" displayFolder="" measureGroup="calls" count="0" oneField="1">
-      <fieldsUsage count="1">
-        <fieldUsage x="4"/>
-      </fieldsUsage>
-    </cacheHierarchy>
-    <cacheHierarchy uniqueName="[Measures].[__XL_Count calls]" caption="__XL_Count calls" measure="1" displayFolder="" measureGroup="calls" count="0" hidden="1"/>
-    <cacheHierarchy uniqueName="[Measures].[__XL_Count customers]" caption="__XL_Count customers" measure="1" displayFolder="" measureGroup="customers" count="0" hidden="1"/>
-    <cacheHierarchy uniqueName="[Measures].[__No measures defined]" caption="__No measures defined" measure="1" displayFolder="" count="0" hidden="1"/>
-    <cacheHierarchy uniqueName="[Measures].[Count of Call number]" caption="Count of Call number" measure="1" displayFolder="" measureGroup="calls" count="0" hidden="1">
-      <extLst>
-        <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{B97F6D7D-B522-45F9-BDA1-12C45D357490}">
-          <x15:cacheHierarchy aggregatedColumn="0"/>
-        </ext>
-      </extLst>
-    </cacheHierarchy>
-  </cacheHierarchies>
-  <kpis count="0"/>
-  <dimensions count="3">
-    <dimension name="calls" uniqueName="[calls]" caption="calls"/>
-    <dimension name="customers" uniqueName="[customers]" caption="customers"/>
-    <dimension measure="1" name="Measures" uniqueName="[Measures]" caption="Measures"/>
-  </dimensions>
-  <measureGroups count="2">
-    <measureGroup name="calls" caption="calls"/>
-    <measureGroup name="customers" caption="customers"/>
-  </measureGroups>
-  <maps count="3">
-    <map measureGroup="0" dimension="0"/>
-    <map measureGroup="0" dimension="1"/>
-    <map measureGroup="1" dimension="1"/>
-  </maps>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{725AE2AE-9491-48be-B2B4-4EB974FC3084}">
-      <x14:pivotCacheDefinition supportSubqueryNonVisual="1" supportSubqueryCalcMem="1" supportAddCalcMems="1"/>
-    </ext>
-  </extLst>
-</pivotCacheDefinition>
-</file>
-
-<file path=xl/pivotCache/pivotCacheDefinition2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" saveData="0" refreshedBy="sivanagajyothi yedururu" refreshedDate="45756.304968402779" backgroundQuery="1" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="0" supportSubquery="1" supportAdvancedDrill="1" xr:uid="{4C5DC1ED-790F-4CA9-92EA-D1B1643E45F8}">
-  <cacheSource type="external" connectionId="2"/>
-  <cacheFields count="3">
-    <cacheField name="[calls].[Representative].[Representative]" caption="Representative" numFmtId="0" hierarchy="3" level="1">
-      <sharedItems count="5">
-        <s v="R01"/>
-        <s v="R02"/>
-        <s v="R03"/>
-        <s v="R04"/>
-        <s v="R05"/>
-      </sharedItems>
-    </cacheField>
-    <cacheField name="[Measures].[call count]" caption="call count" numFmtId="0" hierarchy="17" level="32767"/>
-    <cacheField name="[Measures].[total amount]" caption="total amount" numFmtId="0" hierarchy="18" level="32767"/>
-  </cacheFields>
-  <cacheHierarchies count="26">
-    <cacheHierarchy uniqueName="[calls].[Call number]" caption="Call number" attribute="1" defaultMemberUniqueName="[calls].[Call number].[All]" allUniqueName="[calls].[Call number].[All]" dimensionUniqueName="[calls]" displayFolder="" count="0" memberValueDatatype="130" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[calls].[Customer ID]" caption="Customer ID" attribute="1" defaultMemberUniqueName="[calls].[Customer ID].[All]" allUniqueName="[calls].[Customer ID].[All]" dimensionUniqueName="[calls]" displayFolder="" count="0" memberValueDatatype="130" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[calls].[Duration]" caption="Duration" attribute="1" defaultMemberUniqueName="[calls].[Duration].[All]" allUniqueName="[calls].[Duration].[All]" dimensionUniqueName="[calls]" displayFolder="" count="0" memberValueDatatype="20" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[calls].[Representative]" caption="Representative" attribute="1" defaultMemberUniqueName="[calls].[Representative].[All]" allUniqueName="[calls].[Representative].[All]" dimensionUniqueName="[calls]" displayFolder="" count="2" memberValueDatatype="130" unbalanced="0">
-      <fieldsUsage count="2">
-        <fieldUsage x="-1"/>
-        <fieldUsage x="0"/>
-      </fieldsUsage>
-    </cacheHierarchy>
-    <cacheHierarchy uniqueName="[calls].[Date of Call]" caption="Date of Call" attribute="1" time="1" defaultMemberUniqueName="[calls].[Date of Call].[All]" allUniqueName="[calls].[Date of Call].[All]" dimensionUniqueName="[calls]" displayFolder="" count="0" memberValueDatatype="7" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[calls].[Purchase Amount]" caption="Purchase Amount" attribute="1" defaultMemberUniqueName="[calls].[Purchase Amount].[All]" allUniqueName="[calls].[Purchase Amount].[All]" dimensionUniqueName="[calls]" displayFolder="" count="0" memberValueDatatype="20" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[calls].[Satisfaction Rating]" caption="Satisfaction Rating" attribute="1" defaultMemberUniqueName="[calls].[Satisfaction Rating].[All]" allUniqueName="[calls].[Satisfaction Rating].[All]" dimensionUniqueName="[calls]" displayFolder="" count="0" memberValueDatatype="5" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[calls].[FY]" caption="FY" attribute="1" defaultMemberUniqueName="[calls].[FY].[All]" allUniqueName="[calls].[FY].[All]" dimensionUniqueName="[calls]" displayFolder="" count="0" memberValueDatatype="20" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[calls].[Day of week]" caption="Day of week" attribute="1" defaultMemberUniqueName="[calls].[Day of week].[All]" allUniqueName="[calls].[Day of week].[All]" dimensionUniqueName="[calls]" displayFolder="" count="0" memberValueDatatype="130" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[calls].[Duration Bucket]" caption="Duration Bucket" attribute="1" defaultMemberUniqueName="[calls].[Duration Bucket].[All]" allUniqueName="[calls].[Duration Bucket].[All]" dimensionUniqueName="[calls]" displayFolder="" count="0" memberValueDatatype="130" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[calls].[Rating rounded]" caption="Rating rounded" attribute="1" defaultMemberUniqueName="[calls].[Rating rounded].[All]" allUniqueName="[calls].[Rating rounded].[All]" dimensionUniqueName="[calls]" displayFolder="" count="0" memberValueDatatype="20" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[calls].[Date of Call (Month)]" caption="Date of Call (Month)" attribute="1" defaultMemberUniqueName="[calls].[Date of Call (Month)].[All]" allUniqueName="[calls].[Date of Call (Month)].[All]" dimensionUniqueName="[calls]" displayFolder="" count="0" memberValueDatatype="130" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[customers].[Customer ID]" caption="Customer ID" attribute="1" defaultMemberUniqueName="[customers].[Customer ID].[All]" allUniqueName="[customers].[Customer ID].[All]" dimensionUniqueName="[customers]" displayFolder="" count="0" memberValueDatatype="130" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[customers].[Gedner]" caption="Gedner" attribute="1" defaultMemberUniqueName="[customers].[Gedner].[All]" allUniqueName="[customers].[Gedner].[All]" dimensionUniqueName="[customers]" displayFolder="" count="0" memberValueDatatype="130" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[customers].[Age]" caption="Age" attribute="1" defaultMemberUniqueName="[customers].[Age].[All]" allUniqueName="[customers].[Age].[All]" dimensionUniqueName="[customers]" displayFolder="" count="0" memberValueDatatype="20" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[customers].[City]" caption="City" attribute="1" defaultMemberUniqueName="[customers].[City].[All]" allUniqueName="[customers].[City].[All]" dimensionUniqueName="[customers]" displayFolder="" count="0" memberValueDatatype="130" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[calls].[Date of Call (Month Index)]" caption="Date of Call (Month Index)" attribute="1" defaultMemberUniqueName="[calls].[Date of Call (Month Index)].[All]" allUniqueName="[calls].[Date of Call (Month Index)].[All]" dimensionUniqueName="[calls]" displayFolder="" count="0" memberValueDatatype="20" unbalanced="0" hidden="1"/>
-    <cacheHierarchy uniqueName="[Measures].[call count]" caption="call count" measure="1" displayFolder="" measureGroup="calls" count="0" oneField="1">
-      <fieldsUsage count="1">
-        <fieldUsage x="1"/>
-      </fieldsUsage>
-    </cacheHierarchy>
-    <cacheHierarchy uniqueName="[Measures].[total amount]" caption="total amount" measure="1" displayFolder="" measureGroup="calls" count="0" oneField="1">
-      <fieldsUsage count="1">
-        <fieldUsage x="2"/>
-      </fieldsUsage>
-    </cacheHierarchy>
-    <cacheHierarchy uniqueName="[Measures].[total duration]" caption="total duration" measure="1" displayFolder="" measureGroup="calls" count="0"/>
-    <cacheHierarchy uniqueName="[Measures].[avg rating]" caption="avg rating" measure="1" displayFolder="" measureGroup="calls" count="0"/>
-    <cacheHierarchy uniqueName="[Measures].[5*rating]" caption="5*rating" measure="1" displayFolder="" measureGroup="calls" count="0"/>
-    <cacheHierarchy uniqueName="[Measures].[__XL_Count calls]" caption="__XL_Count calls" measure="1" displayFolder="" measureGroup="calls" count="0" hidden="1"/>
-    <cacheHierarchy uniqueName="[Measures].[__XL_Count customers]" caption="__XL_Count customers" measure="1" displayFolder="" measureGroup="customers" count="0" hidden="1"/>
-    <cacheHierarchy uniqueName="[Measures].[__No measures defined]" caption="__No measures defined" measure="1" displayFolder="" count="0" hidden="1"/>
-    <cacheHierarchy uniqueName="[Measures].[Count of Call number]" caption="Count of Call number" measure="1" displayFolder="" measureGroup="calls" count="0" hidden="1">
-      <extLst>
-        <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{B97F6D7D-B522-45F9-BDA1-12C45D357490}">
-          <x15:cacheHierarchy aggregatedColumn="0"/>
-        </ext>
-      </extLst>
-    </cacheHierarchy>
-  </cacheHierarchies>
-  <kpis count="0"/>
-  <dimensions count="3">
-    <dimension name="calls" uniqueName="[calls]" caption="calls"/>
-    <dimension name="customers" uniqueName="[customers]" caption="customers"/>
-    <dimension measure="1" name="Measures" uniqueName="[Measures]" caption="Measures"/>
-  </dimensions>
-  <measureGroups count="2">
-    <measureGroup name="calls" caption="calls"/>
-    <measureGroup name="customers" caption="customers"/>
-  </measureGroups>
-  <maps count="3">
-    <map measureGroup="0" dimension="0"/>
-    <map measureGroup="0" dimension="1"/>
-    <map measureGroup="1" dimension="1"/>
-  </maps>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{725AE2AE-9491-48be-B2B4-4EB974FC3084}">
-      <x14:pivotCacheDefinition supportSubqueryNonVisual="1" supportSubqueryCalcMem="1" supportAddCalcMems="1"/>
-    </ext>
-  </extLst>
-</pivotCacheDefinition>
-</file>
-
-<file path=xl/pivotCache/pivotCacheDefinition3.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" saveData="0" refreshedBy="sivanagajyothi yedururu" refreshedDate="45756.577913078705" backgroundQuery="1" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="0" supportSubquery="1" supportAdvancedDrill="1" xr:uid="{75F358FF-AB0D-499A-93F7-81A3139FEAE8}">
   <cacheSource type="external" connectionId="2"/>
   <cacheFields count="6">
@@ -13084,7 +12486,7 @@
       <sharedItems containsSemiMixedTypes="0" containsNonDate="0" containsString="0"/>
     </cacheField>
   </cacheFields>
-  <cacheHierarchies count="26">
+  <cacheHierarchies count="27">
     <cacheHierarchy uniqueName="[calls].[Call number]" caption="Call number" attribute="1" defaultMemberUniqueName="[calls].[Call number].[All]" allUniqueName="[calls].[Call number].[All]" dimensionUniqueName="[calls]" displayFolder="" count="0" memberValueDatatype="130" unbalanced="0"/>
     <cacheHierarchy uniqueName="[calls].[Customer ID]" caption="Customer ID" attribute="1" defaultMemberUniqueName="[calls].[Customer ID].[All]" allUniqueName="[calls].[Customer ID].[All]" dimensionUniqueName="[calls]" displayFolder="" count="0" memberValueDatatype="130" unbalanced="0"/>
     <cacheHierarchy uniqueName="[calls].[Duration]" caption="Duration" attribute="1" defaultMemberUniqueName="[calls].[Duration].[All]" allUniqueName="[calls].[Duration].[All]" dimensionUniqueName="[calls]" displayFolder="" count="0" memberValueDatatype="20" unbalanced="0"/>
@@ -13142,6 +12544,186 @@
         </ext>
       </extLst>
     </cacheHierarchy>
+    <cacheHierarchy uniqueName="[Measures].[Count of Gedner]" caption="Count of Gedner" measure="1" displayFolder="" measureGroup="customers" count="0" hidden="1">
+      <extLst>
+        <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{B97F6D7D-B522-45F9-BDA1-12C45D357490}">
+          <x15:cacheHierarchy aggregatedColumn="13"/>
+        </ext>
+      </extLst>
+    </cacheHierarchy>
+  </cacheHierarchies>
+  <kpis count="0"/>
+  <dimensions count="3">
+    <dimension name="calls" uniqueName="[calls]" caption="calls"/>
+    <dimension name="customers" uniqueName="[customers]" caption="customers"/>
+    <dimension measure="1" name="Measures" uniqueName="[Measures]" caption="Measures"/>
+  </dimensions>
+  <measureGroups count="2">
+    <measureGroup name="calls" caption="calls"/>
+    <measureGroup name="customers" caption="customers"/>
+  </measureGroups>
+  <maps count="3">
+    <map measureGroup="0" dimension="0"/>
+    <map measureGroup="0" dimension="1"/>
+    <map measureGroup="1" dimension="1"/>
+  </maps>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{725AE2AE-9491-48be-B2B4-4EB974FC3084}">
+      <x14:pivotCacheDefinition supportSubqueryNonVisual="1" supportSubqueryCalcMem="1" supportAddCalcMems="1"/>
+    </ext>
+  </extLst>
+</pivotCacheDefinition>
+</file>
+
+<file path=xl/pivotCache/pivotCacheDefinition2.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" saveData="0" refreshedBy="sivanagajyothi yedururu" refreshedDate="45755.942241435187" backgroundQuery="1" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="0" supportSubquery="1" supportAdvancedDrill="1" xr:uid="{C9E09126-0EF3-4689-9CCC-21407F27E967}">
+  <cacheSource type="external" connectionId="2"/>
+  <cacheFields count="5">
+    <cacheField name="[Measures].[call count]" caption="call count" numFmtId="0" hierarchy="17" level="32767"/>
+    <cacheField name="[Measures].[total amount]" caption="total amount" numFmtId="0" hierarchy="18" level="32767"/>
+    <cacheField name="[Measures].[total duration]" caption="total duration" numFmtId="0" hierarchy="19" level="32767"/>
+    <cacheField name="[Measures].[avg rating]" caption="avg rating" numFmtId="0" hierarchy="20" level="32767"/>
+    <cacheField name="[Measures].[5*rating]" caption="5*rating" numFmtId="0" hierarchy="21" level="32767"/>
+  </cacheFields>
+  <cacheHierarchies count="27">
+    <cacheHierarchy uniqueName="[calls].[Call number]" caption="Call number" attribute="1" defaultMemberUniqueName="[calls].[Call number].[All]" allUniqueName="[calls].[Call number].[All]" dimensionUniqueName="[calls]" displayFolder="" count="0" memberValueDatatype="130" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[calls].[Customer ID]" caption="Customer ID" attribute="1" defaultMemberUniqueName="[calls].[Customer ID].[All]" allUniqueName="[calls].[Customer ID].[All]" dimensionUniqueName="[calls]" displayFolder="" count="0" memberValueDatatype="130" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[calls].[Duration]" caption="Duration" attribute="1" defaultMemberUniqueName="[calls].[Duration].[All]" allUniqueName="[calls].[Duration].[All]" dimensionUniqueName="[calls]" displayFolder="" count="0" memberValueDatatype="20" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[calls].[Representative]" caption="Representative" attribute="1" defaultMemberUniqueName="[calls].[Representative].[All]" allUniqueName="[calls].[Representative].[All]" dimensionUniqueName="[calls]" displayFolder="" count="0" memberValueDatatype="130" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[calls].[Date of Call]" caption="Date of Call" attribute="1" time="1" defaultMemberUniqueName="[calls].[Date of Call].[All]" allUniqueName="[calls].[Date of Call].[All]" dimensionUniqueName="[calls]" displayFolder="" count="0" memberValueDatatype="7" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[calls].[Purchase Amount]" caption="Purchase Amount" attribute="1" defaultMemberUniqueName="[calls].[Purchase Amount].[All]" allUniqueName="[calls].[Purchase Amount].[All]" dimensionUniqueName="[calls]" displayFolder="" count="0" memberValueDatatype="20" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[calls].[Satisfaction Rating]" caption="Satisfaction Rating" attribute="1" defaultMemberUniqueName="[calls].[Satisfaction Rating].[All]" allUniqueName="[calls].[Satisfaction Rating].[All]" dimensionUniqueName="[calls]" displayFolder="" count="0" memberValueDatatype="5" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[calls].[FY]" caption="FY" attribute="1" defaultMemberUniqueName="[calls].[FY].[All]" allUniqueName="[calls].[FY].[All]" dimensionUniqueName="[calls]" displayFolder="" count="0" memberValueDatatype="20" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[calls].[Day of week]" caption="Day of week" attribute="1" defaultMemberUniqueName="[calls].[Day of week].[All]" allUniqueName="[calls].[Day of week].[All]" dimensionUniqueName="[calls]" displayFolder="" count="0" memberValueDatatype="130" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[calls].[Duration Bucket]" caption="Duration Bucket" attribute="1" defaultMemberUniqueName="[calls].[Duration Bucket].[All]" allUniqueName="[calls].[Duration Bucket].[All]" dimensionUniqueName="[calls]" displayFolder="" count="0" memberValueDatatype="130" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[calls].[Rating rounded]" caption="Rating rounded" attribute="1" defaultMemberUniqueName="[calls].[Rating rounded].[All]" allUniqueName="[calls].[Rating rounded].[All]" dimensionUniqueName="[calls]" displayFolder="" count="0" memberValueDatatype="20" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[calls].[Date of Call (Month)]" caption="Date of Call (Month)" attribute="1" defaultMemberUniqueName="[calls].[Date of Call (Month)].[All]" allUniqueName="[calls].[Date of Call (Month)].[All]" dimensionUniqueName="[calls]" displayFolder="" count="0" memberValueDatatype="130" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[customers].[Customer ID]" caption="Customer ID" attribute="1" defaultMemberUniqueName="[customers].[Customer ID].[All]" allUniqueName="[customers].[Customer ID].[All]" dimensionUniqueName="[customers]" displayFolder="" count="0" memberValueDatatype="130" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[customers].[Gedner]" caption="Gedner" attribute="1" defaultMemberUniqueName="[customers].[Gedner].[All]" allUniqueName="[customers].[Gedner].[All]" dimensionUniqueName="[customers]" displayFolder="" count="0" memberValueDatatype="130" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[customers].[Age]" caption="Age" attribute="1" defaultMemberUniqueName="[customers].[Age].[All]" allUniqueName="[customers].[Age].[All]" dimensionUniqueName="[customers]" displayFolder="" count="0" memberValueDatatype="20" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[customers].[City]" caption="City" attribute="1" defaultMemberUniqueName="[customers].[City].[All]" allUniqueName="[customers].[City].[All]" dimensionUniqueName="[customers]" displayFolder="" count="0" memberValueDatatype="130" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[calls].[Date of Call (Month Index)]" caption="Date of Call (Month Index)" attribute="1" defaultMemberUniqueName="[calls].[Date of Call (Month Index)].[All]" allUniqueName="[calls].[Date of Call (Month Index)].[All]" dimensionUniqueName="[calls]" displayFolder="" count="0" memberValueDatatype="20" unbalanced="0" hidden="1"/>
+    <cacheHierarchy uniqueName="[Measures].[call count]" caption="call count" measure="1" displayFolder="" measureGroup="calls" count="0" oneField="1">
+      <fieldsUsage count="1">
+        <fieldUsage x="0"/>
+      </fieldsUsage>
+    </cacheHierarchy>
+    <cacheHierarchy uniqueName="[Measures].[total amount]" caption="total amount" measure="1" displayFolder="" measureGroup="calls" count="0" oneField="1">
+      <fieldsUsage count="1">
+        <fieldUsage x="1"/>
+      </fieldsUsage>
+    </cacheHierarchy>
+    <cacheHierarchy uniqueName="[Measures].[total duration]" caption="total duration" measure="1" displayFolder="" measureGroup="calls" count="0" oneField="1">
+      <fieldsUsage count="1">
+        <fieldUsage x="2"/>
+      </fieldsUsage>
+    </cacheHierarchy>
+    <cacheHierarchy uniqueName="[Measures].[avg rating]" caption="avg rating" measure="1" displayFolder="" measureGroup="calls" count="0" oneField="1">
+      <fieldsUsage count="1">
+        <fieldUsage x="3"/>
+      </fieldsUsage>
+    </cacheHierarchy>
+    <cacheHierarchy uniqueName="[Measures].[5*rating]" caption="5*rating" measure="1" displayFolder="" measureGroup="calls" count="0" oneField="1">
+      <fieldsUsage count="1">
+        <fieldUsage x="4"/>
+      </fieldsUsage>
+    </cacheHierarchy>
+    <cacheHierarchy uniqueName="[Measures].[__XL_Count calls]" caption="__XL_Count calls" measure="1" displayFolder="" measureGroup="calls" count="0" hidden="1"/>
+    <cacheHierarchy uniqueName="[Measures].[__XL_Count customers]" caption="__XL_Count customers" measure="1" displayFolder="" measureGroup="customers" count="0" hidden="1"/>
+    <cacheHierarchy uniqueName="[Measures].[__No measures defined]" caption="__No measures defined" measure="1" displayFolder="" count="0" hidden="1"/>
+    <cacheHierarchy uniqueName="[Measures].[Count of Call number]" caption="Count of Call number" measure="1" displayFolder="" measureGroup="calls" count="0" hidden="1">
+      <extLst>
+        <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{B97F6D7D-B522-45F9-BDA1-12C45D357490}">
+          <x15:cacheHierarchy aggregatedColumn="0"/>
+        </ext>
+      </extLst>
+    </cacheHierarchy>
+    <cacheHierarchy uniqueName="[Measures].[Count of Gedner]" caption="Count of Gedner" measure="1" displayFolder="" measureGroup="customers" count="0" hidden="1">
+      <extLst>
+        <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{B97F6D7D-B522-45F9-BDA1-12C45D357490}">
+          <x15:cacheHierarchy aggregatedColumn="13"/>
+        </ext>
+      </extLst>
+    </cacheHierarchy>
+  </cacheHierarchies>
+  <kpis count="0"/>
+  <dimensions count="3">
+    <dimension name="calls" uniqueName="[calls]" caption="calls"/>
+    <dimension name="customers" uniqueName="[customers]" caption="customers"/>
+    <dimension measure="1" name="Measures" uniqueName="[Measures]" caption="Measures"/>
+  </dimensions>
+  <measureGroups count="2">
+    <measureGroup name="calls" caption="calls"/>
+    <measureGroup name="customers" caption="customers"/>
+  </measureGroups>
+  <maps count="3">
+    <map measureGroup="0" dimension="0"/>
+    <map measureGroup="0" dimension="1"/>
+    <map measureGroup="1" dimension="1"/>
+  </maps>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{725AE2AE-9491-48be-B2B4-4EB974FC3084}">
+      <x14:pivotCacheDefinition supportSubqueryNonVisual="1" supportSubqueryCalcMem="1" supportAddCalcMems="1"/>
+    </ext>
+  </extLst>
+</pivotCacheDefinition>
+</file>
+
+<file path=xl/pivotCache/pivotCacheDefinition3.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" saveData="0" refreshedBy="sivanagajyothi yedururu" refreshedDate="45756.577914467591" backgroundQuery="1" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="0" supportSubquery="1" supportAdvancedDrill="1" xr:uid="{92373610-BC8A-4D70-A8C7-01427099730D}">
+  <cacheSource type="external" connectionId="2"/>
+  <cacheFields count="1">
+    <cacheField name="[calls].[Representative].[Representative]" caption="Representative" numFmtId="0" hierarchy="3" level="1">
+      <sharedItems count="1">
+        <s v="R05"/>
+      </sharedItems>
+    </cacheField>
+  </cacheFields>
+  <cacheHierarchies count="27">
+    <cacheHierarchy uniqueName="[calls].[Call number]" caption="Call number" attribute="1" defaultMemberUniqueName="[calls].[Call number].[All]" allUniqueName="[calls].[Call number].[All]" dimensionUniqueName="[calls]" displayFolder="" count="0" memberValueDatatype="130" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[calls].[Customer ID]" caption="Customer ID" attribute="1" defaultMemberUniqueName="[calls].[Customer ID].[All]" allUniqueName="[calls].[Customer ID].[All]" dimensionUniqueName="[calls]" displayFolder="" count="0" memberValueDatatype="130" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[calls].[Duration]" caption="Duration" attribute="1" defaultMemberUniqueName="[calls].[Duration].[All]" allUniqueName="[calls].[Duration].[All]" dimensionUniqueName="[calls]" displayFolder="" count="0" memberValueDatatype="20" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[calls].[Representative]" caption="Representative" attribute="1" defaultMemberUniqueName="[calls].[Representative].[All]" allUniqueName="[calls].[Representative].[All]" dimensionUniqueName="[calls]" displayFolder="" count="2" memberValueDatatype="130" unbalanced="0">
+      <fieldsUsage count="2">
+        <fieldUsage x="-1"/>
+        <fieldUsage x="0"/>
+      </fieldsUsage>
+    </cacheHierarchy>
+    <cacheHierarchy uniqueName="[calls].[Date of Call]" caption="Date of Call" attribute="1" time="1" defaultMemberUniqueName="[calls].[Date of Call].[All]" allUniqueName="[calls].[Date of Call].[All]" dimensionUniqueName="[calls]" displayFolder="" count="0" memberValueDatatype="7" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[calls].[Purchase Amount]" caption="Purchase Amount" attribute="1" defaultMemberUniqueName="[calls].[Purchase Amount].[All]" allUniqueName="[calls].[Purchase Amount].[All]" dimensionUniqueName="[calls]" displayFolder="" count="0" memberValueDatatype="20" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[calls].[Satisfaction Rating]" caption="Satisfaction Rating" attribute="1" defaultMemberUniqueName="[calls].[Satisfaction Rating].[All]" allUniqueName="[calls].[Satisfaction Rating].[All]" dimensionUniqueName="[calls]" displayFolder="" count="0" memberValueDatatype="5" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[calls].[FY]" caption="FY" attribute="1" defaultMemberUniqueName="[calls].[FY].[All]" allUniqueName="[calls].[FY].[All]" dimensionUniqueName="[calls]" displayFolder="" count="0" memberValueDatatype="20" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[calls].[Day of week]" caption="Day of week" attribute="1" defaultMemberUniqueName="[calls].[Day of week].[All]" allUniqueName="[calls].[Day of week].[All]" dimensionUniqueName="[calls]" displayFolder="" count="0" memberValueDatatype="130" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[calls].[Duration Bucket]" caption="Duration Bucket" attribute="1" defaultMemberUniqueName="[calls].[Duration Bucket].[All]" allUniqueName="[calls].[Duration Bucket].[All]" dimensionUniqueName="[calls]" displayFolder="" count="0" memberValueDatatype="130" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[calls].[Rating rounded]" caption="Rating rounded" attribute="1" defaultMemberUniqueName="[calls].[Rating rounded].[All]" allUniqueName="[calls].[Rating rounded].[All]" dimensionUniqueName="[calls]" displayFolder="" count="0" memberValueDatatype="20" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[calls].[Date of Call (Month)]" caption="Date of Call (Month)" attribute="1" defaultMemberUniqueName="[calls].[Date of Call (Month)].[All]" allUniqueName="[calls].[Date of Call (Month)].[All]" dimensionUniqueName="[calls]" displayFolder="" count="0" memberValueDatatype="130" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[customers].[Customer ID]" caption="Customer ID" attribute="1" defaultMemberUniqueName="[customers].[Customer ID].[All]" allUniqueName="[customers].[Customer ID].[All]" dimensionUniqueName="[customers]" displayFolder="" count="0" memberValueDatatype="130" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[customers].[Gedner]" caption="Gedner" attribute="1" defaultMemberUniqueName="[customers].[Gedner].[All]" allUniqueName="[customers].[Gedner].[All]" dimensionUniqueName="[customers]" displayFolder="" count="0" memberValueDatatype="130" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[customers].[Age]" caption="Age" attribute="1" defaultMemberUniqueName="[customers].[Age].[All]" allUniqueName="[customers].[Age].[All]" dimensionUniqueName="[customers]" displayFolder="" count="0" memberValueDatatype="20" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[customers].[City]" caption="City" attribute="1" defaultMemberUniqueName="[customers].[City].[All]" allUniqueName="[customers].[City].[All]" dimensionUniqueName="[customers]" displayFolder="" count="0" memberValueDatatype="130" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[calls].[Date of Call (Month Index)]" caption="Date of Call (Month Index)" attribute="1" defaultMemberUniqueName="[calls].[Date of Call (Month Index)].[All]" allUniqueName="[calls].[Date of Call (Month Index)].[All]" dimensionUniqueName="[calls]" displayFolder="" count="0" memberValueDatatype="20" unbalanced="0" hidden="1"/>
+    <cacheHierarchy uniqueName="[Measures].[call count]" caption="call count" measure="1" displayFolder="" measureGroup="calls" count="0"/>
+    <cacheHierarchy uniqueName="[Measures].[total amount]" caption="total amount" measure="1" displayFolder="" measureGroup="calls" count="0"/>
+    <cacheHierarchy uniqueName="[Measures].[total duration]" caption="total duration" measure="1" displayFolder="" measureGroup="calls" count="0"/>
+    <cacheHierarchy uniqueName="[Measures].[avg rating]" caption="avg rating" measure="1" displayFolder="" measureGroup="calls" count="0"/>
+    <cacheHierarchy uniqueName="[Measures].[5*rating]" caption="5*rating" measure="1" displayFolder="" measureGroup="calls" count="0"/>
+    <cacheHierarchy uniqueName="[Measures].[__XL_Count calls]" caption="__XL_Count calls" measure="1" displayFolder="" measureGroup="calls" count="0" hidden="1"/>
+    <cacheHierarchy uniqueName="[Measures].[__XL_Count customers]" caption="__XL_Count customers" measure="1" displayFolder="" measureGroup="customers" count="0" hidden="1"/>
+    <cacheHierarchy uniqueName="[Measures].[__No measures defined]" caption="__No measures defined" measure="1" displayFolder="" count="0" hidden="1"/>
+    <cacheHierarchy uniqueName="[Measures].[Count of Call number]" caption="Count of Call number" measure="1" displayFolder="" measureGroup="calls" count="0" hidden="1">
+      <extLst>
+        <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{B97F6D7D-B522-45F9-BDA1-12C45D357490}">
+          <x15:cacheHierarchy aggregatedColumn="0"/>
+        </ext>
+      </extLst>
+    </cacheHierarchy>
+    <cacheHierarchy uniqueName="[Measures].[Count of Gedner]" caption="Count of Gedner" measure="1" displayFolder="" measureGroup="customers" count="0" hidden="1">
+      <extLst>
+        <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{B97F6D7D-B522-45F9-BDA1-12C45D357490}">
+          <x15:cacheHierarchy aggregatedColumn="13"/>
+        </ext>
+      </extLst>
+    </cacheHierarchy>
   </cacheHierarchies>
   <kpis count="0"/>
   <dimensions count="3">
@@ -13167,6 +12749,197 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition4.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" saveData="0" refreshedBy="sivanagajyothi yedururu" refreshedDate="45756.304968402779" backgroundQuery="1" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="0" supportSubquery="1" supportAdvancedDrill="1" xr:uid="{4C5DC1ED-790F-4CA9-92EA-D1B1643E45F8}">
+  <cacheSource type="external" connectionId="2"/>
+  <cacheFields count="3">
+    <cacheField name="[calls].[Representative].[Representative]" caption="Representative" numFmtId="0" hierarchy="3" level="1">
+      <sharedItems count="5">
+        <s v="R01"/>
+        <s v="R02"/>
+        <s v="R03"/>
+        <s v="R04"/>
+        <s v="R05"/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="[Measures].[call count]" caption="call count" numFmtId="0" hierarchy="17" level="32767"/>
+    <cacheField name="[Measures].[total amount]" caption="total amount" numFmtId="0" hierarchy="18" level="32767"/>
+  </cacheFields>
+  <cacheHierarchies count="27">
+    <cacheHierarchy uniqueName="[calls].[Call number]" caption="Call number" attribute="1" defaultMemberUniqueName="[calls].[Call number].[All]" allUniqueName="[calls].[Call number].[All]" dimensionUniqueName="[calls]" displayFolder="" count="0" memberValueDatatype="130" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[calls].[Customer ID]" caption="Customer ID" attribute="1" defaultMemberUniqueName="[calls].[Customer ID].[All]" allUniqueName="[calls].[Customer ID].[All]" dimensionUniqueName="[calls]" displayFolder="" count="0" memberValueDatatype="130" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[calls].[Duration]" caption="Duration" attribute="1" defaultMemberUniqueName="[calls].[Duration].[All]" allUniqueName="[calls].[Duration].[All]" dimensionUniqueName="[calls]" displayFolder="" count="0" memberValueDatatype="20" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[calls].[Representative]" caption="Representative" attribute="1" defaultMemberUniqueName="[calls].[Representative].[All]" allUniqueName="[calls].[Representative].[All]" dimensionUniqueName="[calls]" displayFolder="" count="2" memberValueDatatype="130" unbalanced="0">
+      <fieldsUsage count="2">
+        <fieldUsage x="-1"/>
+        <fieldUsage x="0"/>
+      </fieldsUsage>
+    </cacheHierarchy>
+    <cacheHierarchy uniqueName="[calls].[Date of Call]" caption="Date of Call" attribute="1" time="1" defaultMemberUniqueName="[calls].[Date of Call].[All]" allUniqueName="[calls].[Date of Call].[All]" dimensionUniqueName="[calls]" displayFolder="" count="0" memberValueDatatype="7" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[calls].[Purchase Amount]" caption="Purchase Amount" attribute="1" defaultMemberUniqueName="[calls].[Purchase Amount].[All]" allUniqueName="[calls].[Purchase Amount].[All]" dimensionUniqueName="[calls]" displayFolder="" count="0" memberValueDatatype="20" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[calls].[Satisfaction Rating]" caption="Satisfaction Rating" attribute="1" defaultMemberUniqueName="[calls].[Satisfaction Rating].[All]" allUniqueName="[calls].[Satisfaction Rating].[All]" dimensionUniqueName="[calls]" displayFolder="" count="0" memberValueDatatype="5" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[calls].[FY]" caption="FY" attribute="1" defaultMemberUniqueName="[calls].[FY].[All]" allUniqueName="[calls].[FY].[All]" dimensionUniqueName="[calls]" displayFolder="" count="0" memberValueDatatype="20" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[calls].[Day of week]" caption="Day of week" attribute="1" defaultMemberUniqueName="[calls].[Day of week].[All]" allUniqueName="[calls].[Day of week].[All]" dimensionUniqueName="[calls]" displayFolder="" count="0" memberValueDatatype="130" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[calls].[Duration Bucket]" caption="Duration Bucket" attribute="1" defaultMemberUniqueName="[calls].[Duration Bucket].[All]" allUniqueName="[calls].[Duration Bucket].[All]" dimensionUniqueName="[calls]" displayFolder="" count="0" memberValueDatatype="130" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[calls].[Rating rounded]" caption="Rating rounded" attribute="1" defaultMemberUniqueName="[calls].[Rating rounded].[All]" allUniqueName="[calls].[Rating rounded].[All]" dimensionUniqueName="[calls]" displayFolder="" count="0" memberValueDatatype="20" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[calls].[Date of Call (Month)]" caption="Date of Call (Month)" attribute="1" defaultMemberUniqueName="[calls].[Date of Call (Month)].[All]" allUniqueName="[calls].[Date of Call (Month)].[All]" dimensionUniqueName="[calls]" displayFolder="" count="0" memberValueDatatype="130" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[customers].[Customer ID]" caption="Customer ID" attribute="1" defaultMemberUniqueName="[customers].[Customer ID].[All]" allUniqueName="[customers].[Customer ID].[All]" dimensionUniqueName="[customers]" displayFolder="" count="0" memberValueDatatype="130" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[customers].[Gedner]" caption="Gedner" attribute="1" defaultMemberUniqueName="[customers].[Gedner].[All]" allUniqueName="[customers].[Gedner].[All]" dimensionUniqueName="[customers]" displayFolder="" count="0" memberValueDatatype="130" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[customers].[Age]" caption="Age" attribute="1" defaultMemberUniqueName="[customers].[Age].[All]" allUniqueName="[customers].[Age].[All]" dimensionUniqueName="[customers]" displayFolder="" count="0" memberValueDatatype="20" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[customers].[City]" caption="City" attribute="1" defaultMemberUniqueName="[customers].[City].[All]" allUniqueName="[customers].[City].[All]" dimensionUniqueName="[customers]" displayFolder="" count="0" memberValueDatatype="130" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[calls].[Date of Call (Month Index)]" caption="Date of Call (Month Index)" attribute="1" defaultMemberUniqueName="[calls].[Date of Call (Month Index)].[All]" allUniqueName="[calls].[Date of Call (Month Index)].[All]" dimensionUniqueName="[calls]" displayFolder="" count="0" memberValueDatatype="20" unbalanced="0" hidden="1"/>
+    <cacheHierarchy uniqueName="[Measures].[call count]" caption="call count" measure="1" displayFolder="" measureGroup="calls" count="0" oneField="1">
+      <fieldsUsage count="1">
+        <fieldUsage x="1"/>
+      </fieldsUsage>
+    </cacheHierarchy>
+    <cacheHierarchy uniqueName="[Measures].[total amount]" caption="total amount" measure="1" displayFolder="" measureGroup="calls" count="0" oneField="1">
+      <fieldsUsage count="1">
+        <fieldUsage x="2"/>
+      </fieldsUsage>
+    </cacheHierarchy>
+    <cacheHierarchy uniqueName="[Measures].[total duration]" caption="total duration" measure="1" displayFolder="" measureGroup="calls" count="0"/>
+    <cacheHierarchy uniqueName="[Measures].[avg rating]" caption="avg rating" measure="1" displayFolder="" measureGroup="calls" count="0"/>
+    <cacheHierarchy uniqueName="[Measures].[5*rating]" caption="5*rating" measure="1" displayFolder="" measureGroup="calls" count="0"/>
+    <cacheHierarchy uniqueName="[Measures].[__XL_Count calls]" caption="__XL_Count calls" measure="1" displayFolder="" measureGroup="calls" count="0" hidden="1"/>
+    <cacheHierarchy uniqueName="[Measures].[__XL_Count customers]" caption="__XL_Count customers" measure="1" displayFolder="" measureGroup="customers" count="0" hidden="1"/>
+    <cacheHierarchy uniqueName="[Measures].[__No measures defined]" caption="__No measures defined" measure="1" displayFolder="" count="0" hidden="1"/>
+    <cacheHierarchy uniqueName="[Measures].[Count of Call number]" caption="Count of Call number" measure="1" displayFolder="" measureGroup="calls" count="0" hidden="1">
+      <extLst>
+        <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{B97F6D7D-B522-45F9-BDA1-12C45D357490}">
+          <x15:cacheHierarchy aggregatedColumn="0"/>
+        </ext>
+      </extLst>
+    </cacheHierarchy>
+    <cacheHierarchy uniqueName="[Measures].[Count of Gedner]" caption="Count of Gedner" measure="1" displayFolder="" measureGroup="customers" count="0" hidden="1">
+      <extLst>
+        <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{B97F6D7D-B522-45F9-BDA1-12C45D357490}">
+          <x15:cacheHierarchy aggregatedColumn="13"/>
+        </ext>
+      </extLst>
+    </cacheHierarchy>
+  </cacheHierarchies>
+  <kpis count="0"/>
+  <dimensions count="3">
+    <dimension name="calls" uniqueName="[calls]" caption="calls"/>
+    <dimension name="customers" uniqueName="[customers]" caption="customers"/>
+    <dimension measure="1" name="Measures" uniqueName="[Measures]" caption="Measures"/>
+  </dimensions>
+  <measureGroups count="2">
+    <measureGroup name="calls" caption="calls"/>
+    <measureGroup name="customers" caption="customers"/>
+  </measureGroups>
+  <maps count="3">
+    <map measureGroup="0" dimension="0"/>
+    <map measureGroup="0" dimension="1"/>
+    <map measureGroup="1" dimension="1"/>
+  </maps>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{725AE2AE-9491-48be-B2B4-4EB974FC3084}">
+      <x14:pivotCacheDefinition supportSubqueryNonVisual="1" supportSubqueryCalcMem="1" supportAddCalcMems="1"/>
+    </ext>
+  </extLst>
+</pivotCacheDefinition>
+</file>
+
+<file path=xl/pivotCache/pivotCacheDefinition5.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" saveData="0" refreshedBy="sivanagajyothi yedururu" refreshedDate="45756.577914120367" backgroundQuery="1" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="0" supportSubquery="1" supportAdvancedDrill="1" xr:uid="{B3312215-48F3-48DA-84C7-101967613022}">
+  <cacheSource type="external" connectionId="2"/>
+  <cacheFields count="3">
+    <cacheField name="[calls].[Representative].[Representative]" caption="Representative" numFmtId="0" hierarchy="3" level="1">
+      <sharedItems containsSemiMixedTypes="0" containsNonDate="0" containsString="0"/>
+    </cacheField>
+    <cacheField name="[calls].[Day of week].[Day of week]" caption="Day of week" numFmtId="0" hierarchy="8" level="1">
+      <sharedItems count="7">
+        <s v="Friday"/>
+        <s v="Monday"/>
+        <s v="Saturday"/>
+        <s v="Sunday"/>
+        <s v="Thursday"/>
+        <s v="Tuesday"/>
+        <s v="Wednesday"/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="[Measures].[call count]" caption="call count" numFmtId="0" hierarchy="17" level="32767"/>
+  </cacheFields>
+  <cacheHierarchies count="27">
+    <cacheHierarchy uniqueName="[calls].[Call number]" caption="Call number" attribute="1" defaultMemberUniqueName="[calls].[Call number].[All]" allUniqueName="[calls].[Call number].[All]" dimensionUniqueName="[calls]" displayFolder="" count="0" memberValueDatatype="130" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[calls].[Customer ID]" caption="Customer ID" attribute="1" defaultMemberUniqueName="[calls].[Customer ID].[All]" allUniqueName="[calls].[Customer ID].[All]" dimensionUniqueName="[calls]" displayFolder="" count="0" memberValueDatatype="130" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[calls].[Duration]" caption="Duration" attribute="1" defaultMemberUniqueName="[calls].[Duration].[All]" allUniqueName="[calls].[Duration].[All]" dimensionUniqueName="[calls]" displayFolder="" count="0" memberValueDatatype="20" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[calls].[Representative]" caption="Representative" attribute="1" defaultMemberUniqueName="[calls].[Representative].[All]" allUniqueName="[calls].[Representative].[All]" dimensionUniqueName="[calls]" displayFolder="" count="2" memberValueDatatype="130" unbalanced="0">
+      <fieldsUsage count="2">
+        <fieldUsage x="-1"/>
+        <fieldUsage x="0"/>
+      </fieldsUsage>
+    </cacheHierarchy>
+    <cacheHierarchy uniqueName="[calls].[Date of Call]" caption="Date of Call" attribute="1" time="1" defaultMemberUniqueName="[calls].[Date of Call].[All]" allUniqueName="[calls].[Date of Call].[All]" dimensionUniqueName="[calls]" displayFolder="" count="0" memberValueDatatype="7" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[calls].[Purchase Amount]" caption="Purchase Amount" attribute="1" defaultMemberUniqueName="[calls].[Purchase Amount].[All]" allUniqueName="[calls].[Purchase Amount].[All]" dimensionUniqueName="[calls]" displayFolder="" count="0" memberValueDatatype="20" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[calls].[Satisfaction Rating]" caption="Satisfaction Rating" attribute="1" defaultMemberUniqueName="[calls].[Satisfaction Rating].[All]" allUniqueName="[calls].[Satisfaction Rating].[All]" dimensionUniqueName="[calls]" displayFolder="" count="0" memberValueDatatype="5" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[calls].[FY]" caption="FY" attribute="1" defaultMemberUniqueName="[calls].[FY].[All]" allUniqueName="[calls].[FY].[All]" dimensionUniqueName="[calls]" displayFolder="" count="0" memberValueDatatype="20" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[calls].[Day of week]" caption="Day of week" attribute="1" defaultMemberUniqueName="[calls].[Day of week].[All]" allUniqueName="[calls].[Day of week].[All]" dimensionUniqueName="[calls]" displayFolder="" count="2" memberValueDatatype="130" unbalanced="0">
+      <fieldsUsage count="2">
+        <fieldUsage x="-1"/>
+        <fieldUsage x="1"/>
+      </fieldsUsage>
+    </cacheHierarchy>
+    <cacheHierarchy uniqueName="[calls].[Duration Bucket]" caption="Duration Bucket" attribute="1" defaultMemberUniqueName="[calls].[Duration Bucket].[All]" allUniqueName="[calls].[Duration Bucket].[All]" dimensionUniqueName="[calls]" displayFolder="" count="0" memberValueDatatype="130" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[calls].[Rating rounded]" caption="Rating rounded" attribute="1" defaultMemberUniqueName="[calls].[Rating rounded].[All]" allUniqueName="[calls].[Rating rounded].[All]" dimensionUniqueName="[calls]" displayFolder="" count="0" memberValueDatatype="20" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[calls].[Date of Call (Month)]" caption="Date of Call (Month)" attribute="1" defaultMemberUniqueName="[calls].[Date of Call (Month)].[All]" allUniqueName="[calls].[Date of Call (Month)].[All]" dimensionUniqueName="[calls]" displayFolder="" count="0" memberValueDatatype="130" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[customers].[Customer ID]" caption="Customer ID" attribute="1" defaultMemberUniqueName="[customers].[Customer ID].[All]" allUniqueName="[customers].[Customer ID].[All]" dimensionUniqueName="[customers]" displayFolder="" count="0" memberValueDatatype="130" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[customers].[Gedner]" caption="Gedner" attribute="1" defaultMemberUniqueName="[customers].[Gedner].[All]" allUniqueName="[customers].[Gedner].[All]" dimensionUniqueName="[customers]" displayFolder="" count="0" memberValueDatatype="130" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[customers].[Age]" caption="Age" attribute="1" defaultMemberUniqueName="[customers].[Age].[All]" allUniqueName="[customers].[Age].[All]" dimensionUniqueName="[customers]" displayFolder="" count="0" memberValueDatatype="20" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[customers].[City]" caption="City" attribute="1" defaultMemberUniqueName="[customers].[City].[All]" allUniqueName="[customers].[City].[All]" dimensionUniqueName="[customers]" displayFolder="" count="0" memberValueDatatype="130" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[calls].[Date of Call (Month Index)]" caption="Date of Call (Month Index)" attribute="1" defaultMemberUniqueName="[calls].[Date of Call (Month Index)].[All]" allUniqueName="[calls].[Date of Call (Month Index)].[All]" dimensionUniqueName="[calls]" displayFolder="" count="0" memberValueDatatype="20" unbalanced="0" hidden="1"/>
+    <cacheHierarchy uniqueName="[Measures].[call count]" caption="call count" measure="1" displayFolder="" measureGroup="calls" count="0" oneField="1">
+      <fieldsUsage count="1">
+        <fieldUsage x="2"/>
+      </fieldsUsage>
+    </cacheHierarchy>
+    <cacheHierarchy uniqueName="[Measures].[total amount]" caption="total amount" measure="1" displayFolder="" measureGroup="calls" count="0"/>
+    <cacheHierarchy uniqueName="[Measures].[total duration]" caption="total duration" measure="1" displayFolder="" measureGroup="calls" count="0"/>
+    <cacheHierarchy uniqueName="[Measures].[avg rating]" caption="avg rating" measure="1" displayFolder="" measureGroup="calls" count="0"/>
+    <cacheHierarchy uniqueName="[Measures].[5*rating]" caption="5*rating" measure="1" displayFolder="" measureGroup="calls" count="0"/>
+    <cacheHierarchy uniqueName="[Measures].[__XL_Count calls]" caption="__XL_Count calls" measure="1" displayFolder="" measureGroup="calls" count="0" hidden="1"/>
+    <cacheHierarchy uniqueName="[Measures].[__XL_Count customers]" caption="__XL_Count customers" measure="1" displayFolder="" measureGroup="customers" count="0" hidden="1"/>
+    <cacheHierarchy uniqueName="[Measures].[__No measures defined]" caption="__No measures defined" measure="1" displayFolder="" count="0" hidden="1"/>
+    <cacheHierarchy uniqueName="[Measures].[Count of Call number]" caption="Count of Call number" measure="1" displayFolder="" measureGroup="calls" count="0" hidden="1">
+      <extLst>
+        <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{B97F6D7D-B522-45F9-BDA1-12C45D357490}">
+          <x15:cacheHierarchy aggregatedColumn="0"/>
+        </ext>
+      </extLst>
+    </cacheHierarchy>
+    <cacheHierarchy uniqueName="[Measures].[Count of Gedner]" caption="Count of Gedner" measure="1" displayFolder="" measureGroup="customers" count="0" hidden="1">
+      <extLst>
+        <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{B97F6D7D-B522-45F9-BDA1-12C45D357490}">
+          <x15:cacheHierarchy aggregatedColumn="13"/>
+        </ext>
+      </extLst>
+    </cacheHierarchy>
+  </cacheHierarchies>
+  <kpis count="0"/>
+  <dimensions count="3">
+    <dimension name="calls" uniqueName="[calls]" caption="calls"/>
+    <dimension name="customers" uniqueName="[customers]" caption="customers"/>
+    <dimension measure="1" name="Measures" uniqueName="[Measures]" caption="Measures"/>
+  </dimensions>
+  <measureGroups count="2">
+    <measureGroup name="calls" caption="calls"/>
+    <measureGroup name="customers" caption="customers"/>
+  </measureGroups>
+  <maps count="3">
+    <map measureGroup="0" dimension="0"/>
+    <map measureGroup="0" dimension="1"/>
+    <map measureGroup="1" dimension="1"/>
+  </maps>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{725AE2AE-9491-48be-B2B4-4EB974FC3084}">
+      <x14:pivotCacheDefinition supportSubqueryNonVisual="1" supportSubqueryCalcMem="1" supportAddCalcMems="1"/>
+    </ext>
+  </extLst>
+</pivotCacheDefinition>
+</file>
+
+<file path=xl/pivotCache/pivotCacheDefinition6.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" saveData="0" refreshedBy="sivanagajyothi yedururu" refreshedDate="45756.577913657406" backgroundQuery="1" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="0" supportSubquery="1" supportAdvancedDrill="1" xr:uid="{5159991F-E602-45B4-B5A0-E05043722C99}">
   <cacheSource type="external" connectionId="2"/>
   <cacheFields count="5">
@@ -13354,7 +13127,7 @@
     <cacheField name="[Measures].[Count of Call number]" caption="Count of Call number" numFmtId="0" hierarchy="25" level="32767"/>
     <cacheField name="[Measures].[call count]" caption="call count" numFmtId="0" hierarchy="17" level="32767"/>
   </cacheFields>
-  <cacheHierarchies count="26">
+  <cacheHierarchies count="27">
     <cacheHierarchy uniqueName="[calls].[Call number]" caption="Call number" attribute="1" defaultMemberUniqueName="[calls].[Call number].[All]" allUniqueName="[calls].[Call number].[All]" dimensionUniqueName="[calls]" displayFolder="" count="0" memberValueDatatype="130" unbalanced="0"/>
     <cacheHierarchy uniqueName="[calls].[Customer ID]" caption="Customer ID" attribute="1" defaultMemberUniqueName="[calls].[Customer ID].[All]" allUniqueName="[calls].[Customer ID].[All]" dimensionUniqueName="[calls]" displayFolder="" count="0" memberValueDatatype="130" unbalanced="0"/>
     <cacheHierarchy uniqueName="[calls].[Duration]" caption="Duration" attribute="1" defaultMemberUniqueName="[calls].[Duration].[All]" allUniqueName="[calls].[Duration].[All]" dimensionUniqueName="[calls]" displayFolder="" count="0" memberValueDatatype="20" unbalanced="0"/>
@@ -13409,166 +13182,10 @@
         </ext>
       </extLst>
     </cacheHierarchy>
-  </cacheHierarchies>
-  <kpis count="0"/>
-  <dimensions count="3">
-    <dimension name="calls" uniqueName="[calls]" caption="calls"/>
-    <dimension name="customers" uniqueName="[customers]" caption="customers"/>
-    <dimension measure="1" name="Measures" uniqueName="[Measures]" caption="Measures"/>
-  </dimensions>
-  <measureGroups count="2">
-    <measureGroup name="calls" caption="calls"/>
-    <measureGroup name="customers" caption="customers"/>
-  </measureGroups>
-  <maps count="3">
-    <map measureGroup="0" dimension="0"/>
-    <map measureGroup="0" dimension="1"/>
-    <map measureGroup="1" dimension="1"/>
-  </maps>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{725AE2AE-9491-48be-B2B4-4EB974FC3084}">
-      <x14:pivotCacheDefinition supportSubqueryNonVisual="1" supportSubqueryCalcMem="1" supportAddCalcMems="1"/>
-    </ext>
-  </extLst>
-</pivotCacheDefinition>
-</file>
-
-<file path=xl/pivotCache/pivotCacheDefinition5.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" saveData="0" refreshedBy="sivanagajyothi yedururu" refreshedDate="45756.577914120367" backgroundQuery="1" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="0" supportSubquery="1" supportAdvancedDrill="1" xr:uid="{B3312215-48F3-48DA-84C7-101967613022}">
-  <cacheSource type="external" connectionId="2"/>
-  <cacheFields count="3">
-    <cacheField name="[calls].[Representative].[Representative]" caption="Representative" numFmtId="0" hierarchy="3" level="1">
-      <sharedItems containsSemiMixedTypes="0" containsNonDate="0" containsString="0"/>
-    </cacheField>
-    <cacheField name="[calls].[Day of week].[Day of week]" caption="Day of week" numFmtId="0" hierarchy="8" level="1">
-      <sharedItems count="7">
-        <s v="Friday"/>
-        <s v="Monday"/>
-        <s v="Saturday"/>
-        <s v="Sunday"/>
-        <s v="Thursday"/>
-        <s v="Tuesday"/>
-        <s v="Wednesday"/>
-      </sharedItems>
-    </cacheField>
-    <cacheField name="[Measures].[call count]" caption="call count" numFmtId="0" hierarchy="17" level="32767"/>
-  </cacheFields>
-  <cacheHierarchies count="26">
-    <cacheHierarchy uniqueName="[calls].[Call number]" caption="Call number" attribute="1" defaultMemberUniqueName="[calls].[Call number].[All]" allUniqueName="[calls].[Call number].[All]" dimensionUniqueName="[calls]" displayFolder="" count="0" memberValueDatatype="130" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[calls].[Customer ID]" caption="Customer ID" attribute="1" defaultMemberUniqueName="[calls].[Customer ID].[All]" allUniqueName="[calls].[Customer ID].[All]" dimensionUniqueName="[calls]" displayFolder="" count="0" memberValueDatatype="130" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[calls].[Duration]" caption="Duration" attribute="1" defaultMemberUniqueName="[calls].[Duration].[All]" allUniqueName="[calls].[Duration].[All]" dimensionUniqueName="[calls]" displayFolder="" count="0" memberValueDatatype="20" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[calls].[Representative]" caption="Representative" attribute="1" defaultMemberUniqueName="[calls].[Representative].[All]" allUniqueName="[calls].[Representative].[All]" dimensionUniqueName="[calls]" displayFolder="" count="2" memberValueDatatype="130" unbalanced="0">
-      <fieldsUsage count="2">
-        <fieldUsage x="-1"/>
-        <fieldUsage x="0"/>
-      </fieldsUsage>
-    </cacheHierarchy>
-    <cacheHierarchy uniqueName="[calls].[Date of Call]" caption="Date of Call" attribute="1" time="1" defaultMemberUniqueName="[calls].[Date of Call].[All]" allUniqueName="[calls].[Date of Call].[All]" dimensionUniqueName="[calls]" displayFolder="" count="2" memberValueDatatype="7" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[calls].[Purchase Amount]" caption="Purchase Amount" attribute="1" defaultMemberUniqueName="[calls].[Purchase Amount].[All]" allUniqueName="[calls].[Purchase Amount].[All]" dimensionUniqueName="[calls]" displayFolder="" count="0" memberValueDatatype="20" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[calls].[Satisfaction Rating]" caption="Satisfaction Rating" attribute="1" defaultMemberUniqueName="[calls].[Satisfaction Rating].[All]" allUniqueName="[calls].[Satisfaction Rating].[All]" dimensionUniqueName="[calls]" displayFolder="" count="0" memberValueDatatype="5" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[calls].[FY]" caption="FY" attribute="1" defaultMemberUniqueName="[calls].[FY].[All]" allUniqueName="[calls].[FY].[All]" dimensionUniqueName="[calls]" displayFolder="" count="0" memberValueDatatype="20" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[calls].[Day of week]" caption="Day of week" attribute="1" defaultMemberUniqueName="[calls].[Day of week].[All]" allUniqueName="[calls].[Day of week].[All]" dimensionUniqueName="[calls]" displayFolder="" count="2" memberValueDatatype="130" unbalanced="0">
-      <fieldsUsage count="2">
-        <fieldUsage x="-1"/>
-        <fieldUsage x="1"/>
-      </fieldsUsage>
-    </cacheHierarchy>
-    <cacheHierarchy uniqueName="[calls].[Duration Bucket]" caption="Duration Bucket" attribute="1" defaultMemberUniqueName="[calls].[Duration Bucket].[All]" allUniqueName="[calls].[Duration Bucket].[All]" dimensionUniqueName="[calls]" displayFolder="" count="0" memberValueDatatype="130" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[calls].[Rating rounded]" caption="Rating rounded" attribute="1" defaultMemberUniqueName="[calls].[Rating rounded].[All]" allUniqueName="[calls].[Rating rounded].[All]" dimensionUniqueName="[calls]" displayFolder="" count="0" memberValueDatatype="20" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[calls].[Date of Call (Month)]" caption="Date of Call (Month)" attribute="1" defaultMemberUniqueName="[calls].[Date of Call (Month)].[All]" allUniqueName="[calls].[Date of Call (Month)].[All]" dimensionUniqueName="[calls]" displayFolder="" count="2" memberValueDatatype="130" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[customers].[Customer ID]" caption="Customer ID" attribute="1" defaultMemberUniqueName="[customers].[Customer ID].[All]" allUniqueName="[customers].[Customer ID].[All]" dimensionUniqueName="[customers]" displayFolder="" count="0" memberValueDatatype="130" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[customers].[Gedner]" caption="Gedner" attribute="1" defaultMemberUniqueName="[customers].[Gedner].[All]" allUniqueName="[customers].[Gedner].[All]" dimensionUniqueName="[customers]" displayFolder="" count="0" memberValueDatatype="130" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[customers].[Age]" caption="Age" attribute="1" defaultMemberUniqueName="[customers].[Age].[All]" allUniqueName="[customers].[Age].[All]" dimensionUniqueName="[customers]" displayFolder="" count="0" memberValueDatatype="20" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[customers].[City]" caption="City" attribute="1" defaultMemberUniqueName="[customers].[City].[All]" allUniqueName="[customers].[City].[All]" dimensionUniqueName="[customers]" displayFolder="" count="0" memberValueDatatype="130" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[calls].[Date of Call (Month Index)]" caption="Date of Call (Month Index)" attribute="1" defaultMemberUniqueName="[calls].[Date of Call (Month Index)].[All]" allUniqueName="[calls].[Date of Call (Month Index)].[All]" dimensionUniqueName="[calls]" displayFolder="" count="0" memberValueDatatype="20" unbalanced="0" hidden="1"/>
-    <cacheHierarchy uniqueName="[Measures].[call count]" caption="call count" measure="1" displayFolder="" measureGroup="calls" count="0" oneField="1">
-      <fieldsUsage count="1">
-        <fieldUsage x="2"/>
-      </fieldsUsage>
-    </cacheHierarchy>
-    <cacheHierarchy uniqueName="[Measures].[total amount]" caption="total amount" measure="1" displayFolder="" measureGroup="calls" count="0"/>
-    <cacheHierarchy uniqueName="[Measures].[total duration]" caption="total duration" measure="1" displayFolder="" measureGroup="calls" count="0"/>
-    <cacheHierarchy uniqueName="[Measures].[avg rating]" caption="avg rating" measure="1" displayFolder="" measureGroup="calls" count="0"/>
-    <cacheHierarchy uniqueName="[Measures].[5*rating]" caption="5*rating" measure="1" displayFolder="" measureGroup="calls" count="0"/>
-    <cacheHierarchy uniqueName="[Measures].[__XL_Count calls]" caption="__XL_Count calls" measure="1" displayFolder="" measureGroup="calls" count="0" hidden="1"/>
-    <cacheHierarchy uniqueName="[Measures].[__XL_Count customers]" caption="__XL_Count customers" measure="1" displayFolder="" measureGroup="customers" count="0" hidden="1"/>
-    <cacheHierarchy uniqueName="[Measures].[__No measures defined]" caption="__No measures defined" measure="1" displayFolder="" count="0" hidden="1"/>
-    <cacheHierarchy uniqueName="[Measures].[Count of Call number]" caption="Count of Call number" measure="1" displayFolder="" measureGroup="calls" count="0" hidden="1">
+    <cacheHierarchy uniqueName="[Measures].[Count of Gedner]" caption="Count of Gedner" measure="1" displayFolder="" measureGroup="customers" count="0" hidden="1">
       <extLst>
         <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{B97F6D7D-B522-45F9-BDA1-12C45D357490}">
-          <x15:cacheHierarchy aggregatedColumn="0"/>
-        </ext>
-      </extLst>
-    </cacheHierarchy>
-  </cacheHierarchies>
-  <kpis count="0"/>
-  <dimensions count="3">
-    <dimension name="calls" uniqueName="[calls]" caption="calls"/>
-    <dimension name="customers" uniqueName="[customers]" caption="customers"/>
-    <dimension measure="1" name="Measures" uniqueName="[Measures]" caption="Measures"/>
-  </dimensions>
-  <measureGroups count="2">
-    <measureGroup name="calls" caption="calls"/>
-    <measureGroup name="customers" caption="customers"/>
-  </measureGroups>
-  <maps count="3">
-    <map measureGroup="0" dimension="0"/>
-    <map measureGroup="0" dimension="1"/>
-    <map measureGroup="1" dimension="1"/>
-  </maps>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{725AE2AE-9491-48be-B2B4-4EB974FC3084}">
-      <x14:pivotCacheDefinition supportSubqueryNonVisual="1" supportSubqueryCalcMem="1" supportAddCalcMems="1"/>
-    </ext>
-  </extLst>
-</pivotCacheDefinition>
-</file>
-
-<file path=xl/pivotCache/pivotCacheDefinition6.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" saveData="0" refreshedBy="sivanagajyothi yedururu" refreshedDate="45756.577914467591" backgroundQuery="1" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="0" supportSubquery="1" supportAdvancedDrill="1" xr:uid="{92373610-BC8A-4D70-A8C7-01427099730D}">
-  <cacheSource type="external" connectionId="2"/>
-  <cacheFields count="1">
-    <cacheField name="[calls].[Representative].[Representative]" caption="Representative" numFmtId="0" hierarchy="3" level="1">
-      <sharedItems count="1">
-        <s v="R05"/>
-      </sharedItems>
-    </cacheField>
-  </cacheFields>
-  <cacheHierarchies count="26">
-    <cacheHierarchy uniqueName="[calls].[Call number]" caption="Call number" attribute="1" defaultMemberUniqueName="[calls].[Call number].[All]" allUniqueName="[calls].[Call number].[All]" dimensionUniqueName="[calls]" displayFolder="" count="0" memberValueDatatype="130" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[calls].[Customer ID]" caption="Customer ID" attribute="1" defaultMemberUniqueName="[calls].[Customer ID].[All]" allUniqueName="[calls].[Customer ID].[All]" dimensionUniqueName="[calls]" displayFolder="" count="0" memberValueDatatype="130" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[calls].[Duration]" caption="Duration" attribute="1" defaultMemberUniqueName="[calls].[Duration].[All]" allUniqueName="[calls].[Duration].[All]" dimensionUniqueName="[calls]" displayFolder="" count="0" memberValueDatatype="20" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[calls].[Representative]" caption="Representative" attribute="1" defaultMemberUniqueName="[calls].[Representative].[All]" allUniqueName="[calls].[Representative].[All]" dimensionUniqueName="[calls]" displayFolder="" count="2" memberValueDatatype="130" unbalanced="0">
-      <fieldsUsage count="2">
-        <fieldUsage x="-1"/>
-        <fieldUsage x="0"/>
-      </fieldsUsage>
-    </cacheHierarchy>
-    <cacheHierarchy uniqueName="[calls].[Date of Call]" caption="Date of Call" attribute="1" time="1" defaultMemberUniqueName="[calls].[Date of Call].[All]" allUniqueName="[calls].[Date of Call].[All]" dimensionUniqueName="[calls]" displayFolder="" count="0" memberValueDatatype="7" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[calls].[Purchase Amount]" caption="Purchase Amount" attribute="1" defaultMemberUniqueName="[calls].[Purchase Amount].[All]" allUniqueName="[calls].[Purchase Amount].[All]" dimensionUniqueName="[calls]" displayFolder="" count="0" memberValueDatatype="20" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[calls].[Satisfaction Rating]" caption="Satisfaction Rating" attribute="1" defaultMemberUniqueName="[calls].[Satisfaction Rating].[All]" allUniqueName="[calls].[Satisfaction Rating].[All]" dimensionUniqueName="[calls]" displayFolder="" count="0" memberValueDatatype="5" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[calls].[FY]" caption="FY" attribute="1" defaultMemberUniqueName="[calls].[FY].[All]" allUniqueName="[calls].[FY].[All]" dimensionUniqueName="[calls]" displayFolder="" count="0" memberValueDatatype="20" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[calls].[Day of week]" caption="Day of week" attribute="1" defaultMemberUniqueName="[calls].[Day of week].[All]" allUniqueName="[calls].[Day of week].[All]" dimensionUniqueName="[calls]" displayFolder="" count="0" memberValueDatatype="130" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[calls].[Duration Bucket]" caption="Duration Bucket" attribute="1" defaultMemberUniqueName="[calls].[Duration Bucket].[All]" allUniqueName="[calls].[Duration Bucket].[All]" dimensionUniqueName="[calls]" displayFolder="" count="0" memberValueDatatype="130" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[calls].[Rating rounded]" caption="Rating rounded" attribute="1" defaultMemberUniqueName="[calls].[Rating rounded].[All]" allUniqueName="[calls].[Rating rounded].[All]" dimensionUniqueName="[calls]" displayFolder="" count="0" memberValueDatatype="20" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[calls].[Date of Call (Month)]" caption="Date of Call (Month)" attribute="1" defaultMemberUniqueName="[calls].[Date of Call (Month)].[All]" allUniqueName="[calls].[Date of Call (Month)].[All]" dimensionUniqueName="[calls]" displayFolder="" count="0" memberValueDatatype="130" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[customers].[Customer ID]" caption="Customer ID" attribute="1" defaultMemberUniqueName="[customers].[Customer ID].[All]" allUniqueName="[customers].[Customer ID].[All]" dimensionUniqueName="[customers]" displayFolder="" count="0" memberValueDatatype="130" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[customers].[Gedner]" caption="Gedner" attribute="1" defaultMemberUniqueName="[customers].[Gedner].[All]" allUniqueName="[customers].[Gedner].[All]" dimensionUniqueName="[customers]" displayFolder="" count="0" memberValueDatatype="130" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[customers].[Age]" caption="Age" attribute="1" defaultMemberUniqueName="[customers].[Age].[All]" allUniqueName="[customers].[Age].[All]" dimensionUniqueName="[customers]" displayFolder="" count="0" memberValueDatatype="20" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[customers].[City]" caption="City" attribute="1" defaultMemberUniqueName="[customers].[City].[All]" allUniqueName="[customers].[City].[All]" dimensionUniqueName="[customers]" displayFolder="" count="0" memberValueDatatype="130" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[calls].[Date of Call (Month Index)]" caption="Date of Call (Month Index)" attribute="1" defaultMemberUniqueName="[calls].[Date of Call (Month Index)].[All]" allUniqueName="[calls].[Date of Call (Month Index)].[All]" dimensionUniqueName="[calls]" displayFolder="" count="0" memberValueDatatype="20" unbalanced="0" hidden="1"/>
-    <cacheHierarchy uniqueName="[Measures].[call count]" caption="call count" measure="1" displayFolder="" measureGroup="calls" count="0"/>
-    <cacheHierarchy uniqueName="[Measures].[total amount]" caption="total amount" measure="1" displayFolder="" measureGroup="calls" count="0"/>
-    <cacheHierarchy uniqueName="[Measures].[total duration]" caption="total duration" measure="1" displayFolder="" measureGroup="calls" count="0"/>
-    <cacheHierarchy uniqueName="[Measures].[avg rating]" caption="avg rating" measure="1" displayFolder="" measureGroup="calls" count="0"/>
-    <cacheHierarchy uniqueName="[Measures].[5*rating]" caption="5*rating" measure="1" displayFolder="" measureGroup="calls" count="0"/>
-    <cacheHierarchy uniqueName="[Measures].[__XL_Count calls]" caption="__XL_Count calls" measure="1" displayFolder="" measureGroup="calls" count="0" hidden="1"/>
-    <cacheHierarchy uniqueName="[Measures].[__XL_Count customers]" caption="__XL_Count customers" measure="1" displayFolder="" measureGroup="customers" count="0" hidden="1"/>
-    <cacheHierarchy uniqueName="[Measures].[__No measures defined]" caption="__No measures defined" measure="1" displayFolder="" count="0" hidden="1"/>
-    <cacheHierarchy uniqueName="[Measures].[Count of Call number]" caption="Count of Call number" measure="1" displayFolder="" measureGroup="calls" count="0" hidden="1">
-      <extLst>
-        <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{B97F6D7D-B522-45F9-BDA1-12C45D357490}">
-          <x15:cacheHierarchy aggregatedColumn="0"/>
+          <x15:cacheHierarchy aggregatedColumn="13"/>
         </ext>
       </extLst>
     </cacheHierarchy>
@@ -13597,6 +13214,103 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition7.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" saveData="0" refreshedBy="sivanagajyothi yedururu" refreshedDate="45756.80612789352" backgroundQuery="1" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="0" supportSubquery="1" supportAdvancedDrill="1" xr:uid="{D37CFB76-E8AE-422E-B253-C7AC9F821EAC}">
+  <cacheSource type="external" connectionId="2"/>
+  <cacheFields count="3">
+    <cacheField name="[customers].[City].[City]" caption="City" numFmtId="0" hierarchy="15" level="1">
+      <sharedItems count="3">
+        <s v="Cincinnati"/>
+        <s v="Cleveland"/>
+        <s v="Columbus"/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="[customers].[Gedner].[Gedner]" caption="Gedner" numFmtId="0" hierarchy="13" level="1">
+      <sharedItems count="2">
+        <s v="Female"/>
+        <s v="Male"/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="[Measures].[call count]" caption="call count" numFmtId="0" hierarchy="17" level="32767"/>
+  </cacheFields>
+  <cacheHierarchies count="27">
+    <cacheHierarchy uniqueName="[calls].[Call number]" caption="Call number" attribute="1" defaultMemberUniqueName="[calls].[Call number].[All]" allUniqueName="[calls].[Call number].[All]" dimensionUniqueName="[calls]" displayFolder="" count="0" memberValueDatatype="130" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[calls].[Customer ID]" caption="Customer ID" attribute="1" defaultMemberUniqueName="[calls].[Customer ID].[All]" allUniqueName="[calls].[Customer ID].[All]" dimensionUniqueName="[calls]" displayFolder="" count="0" memberValueDatatype="130" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[calls].[Duration]" caption="Duration" attribute="1" defaultMemberUniqueName="[calls].[Duration].[All]" allUniqueName="[calls].[Duration].[All]" dimensionUniqueName="[calls]" displayFolder="" count="0" memberValueDatatype="20" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[calls].[Representative]" caption="Representative" attribute="1" defaultMemberUniqueName="[calls].[Representative].[All]" allUniqueName="[calls].[Representative].[All]" dimensionUniqueName="[calls]" displayFolder="" count="0" memberValueDatatype="130" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[calls].[Date of Call]" caption="Date of Call" attribute="1" time="1" defaultMemberUniqueName="[calls].[Date of Call].[All]" allUniqueName="[calls].[Date of Call].[All]" dimensionUniqueName="[calls]" displayFolder="" count="0" memberValueDatatype="7" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[calls].[Purchase Amount]" caption="Purchase Amount" attribute="1" defaultMemberUniqueName="[calls].[Purchase Amount].[All]" allUniqueName="[calls].[Purchase Amount].[All]" dimensionUniqueName="[calls]" displayFolder="" count="0" memberValueDatatype="20" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[calls].[Satisfaction Rating]" caption="Satisfaction Rating" attribute="1" defaultMemberUniqueName="[calls].[Satisfaction Rating].[All]" allUniqueName="[calls].[Satisfaction Rating].[All]" dimensionUniqueName="[calls]" displayFolder="" count="0" memberValueDatatype="5" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[calls].[FY]" caption="FY" attribute="1" defaultMemberUniqueName="[calls].[FY].[All]" allUniqueName="[calls].[FY].[All]" dimensionUniqueName="[calls]" displayFolder="" count="0" memberValueDatatype="20" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[calls].[Day of week]" caption="Day of week" attribute="1" defaultMemberUniqueName="[calls].[Day of week].[All]" allUniqueName="[calls].[Day of week].[All]" dimensionUniqueName="[calls]" displayFolder="" count="0" memberValueDatatype="130" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[calls].[Duration Bucket]" caption="Duration Bucket" attribute="1" defaultMemberUniqueName="[calls].[Duration Bucket].[All]" allUniqueName="[calls].[Duration Bucket].[All]" dimensionUniqueName="[calls]" displayFolder="" count="0" memberValueDatatype="130" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[calls].[Rating rounded]" caption="Rating rounded" attribute="1" defaultMemberUniqueName="[calls].[Rating rounded].[All]" allUniqueName="[calls].[Rating rounded].[All]" dimensionUniqueName="[calls]" displayFolder="" count="0" memberValueDatatype="20" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[calls].[Date of Call (Month)]" caption="Date of Call (Month)" attribute="1" defaultMemberUniqueName="[calls].[Date of Call (Month)].[All]" allUniqueName="[calls].[Date of Call (Month)].[All]" dimensionUniqueName="[calls]" displayFolder="" count="0" memberValueDatatype="130" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[customers].[Customer ID]" caption="Customer ID" attribute="1" defaultMemberUniqueName="[customers].[Customer ID].[All]" allUniqueName="[customers].[Customer ID].[All]" dimensionUniqueName="[customers]" displayFolder="" count="0" memberValueDatatype="130" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[customers].[Gedner]" caption="Gedner" attribute="1" defaultMemberUniqueName="[customers].[Gedner].[All]" allUniqueName="[customers].[Gedner].[All]" dimensionUniqueName="[customers]" displayFolder="" count="2" memberValueDatatype="130" unbalanced="0">
+      <fieldsUsage count="2">
+        <fieldUsage x="-1"/>
+        <fieldUsage x="1"/>
+      </fieldsUsage>
+    </cacheHierarchy>
+    <cacheHierarchy uniqueName="[customers].[Age]" caption="Age" attribute="1" defaultMemberUniqueName="[customers].[Age].[All]" allUniqueName="[customers].[Age].[All]" dimensionUniqueName="[customers]" displayFolder="" count="0" memberValueDatatype="20" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[customers].[City]" caption="City" attribute="1" defaultMemberUniqueName="[customers].[City].[All]" allUniqueName="[customers].[City].[All]" dimensionUniqueName="[customers]" displayFolder="" count="2" memberValueDatatype="130" unbalanced="0">
+      <fieldsUsage count="2">
+        <fieldUsage x="-1"/>
+        <fieldUsage x="0"/>
+      </fieldsUsage>
+    </cacheHierarchy>
+    <cacheHierarchy uniqueName="[calls].[Date of Call (Month Index)]" caption="Date of Call (Month Index)" attribute="1" defaultMemberUniqueName="[calls].[Date of Call (Month Index)].[All]" allUniqueName="[calls].[Date of Call (Month Index)].[All]" dimensionUniqueName="[calls]" displayFolder="" count="0" memberValueDatatype="20" unbalanced="0" hidden="1"/>
+    <cacheHierarchy uniqueName="[Measures].[call count]" caption="call count" measure="1" displayFolder="" measureGroup="calls" count="0" oneField="1">
+      <fieldsUsage count="1">
+        <fieldUsage x="2"/>
+      </fieldsUsage>
+    </cacheHierarchy>
+    <cacheHierarchy uniqueName="[Measures].[total amount]" caption="total amount" measure="1" displayFolder="" measureGroup="calls" count="0"/>
+    <cacheHierarchy uniqueName="[Measures].[total duration]" caption="total duration" measure="1" displayFolder="" measureGroup="calls" count="0"/>
+    <cacheHierarchy uniqueName="[Measures].[avg rating]" caption="avg rating" measure="1" displayFolder="" measureGroup="calls" count="0"/>
+    <cacheHierarchy uniqueName="[Measures].[5*rating]" caption="5*rating" measure="1" displayFolder="" measureGroup="calls" count="0"/>
+    <cacheHierarchy uniqueName="[Measures].[__XL_Count calls]" caption="__XL_Count calls" measure="1" displayFolder="" measureGroup="calls" count="0" hidden="1"/>
+    <cacheHierarchy uniqueName="[Measures].[__XL_Count customers]" caption="__XL_Count customers" measure="1" displayFolder="" measureGroup="customers" count="0" hidden="1"/>
+    <cacheHierarchy uniqueName="[Measures].[__No measures defined]" caption="__No measures defined" measure="1" displayFolder="" count="0" hidden="1"/>
+    <cacheHierarchy uniqueName="[Measures].[Count of Call number]" caption="Count of Call number" measure="1" displayFolder="" measureGroup="calls" count="0" hidden="1">
+      <extLst>
+        <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{B97F6D7D-B522-45F9-BDA1-12C45D357490}">
+          <x15:cacheHierarchy aggregatedColumn="0"/>
+        </ext>
+      </extLst>
+    </cacheHierarchy>
+    <cacheHierarchy uniqueName="[Measures].[Count of Gedner]" caption="Count of Gedner" measure="1" displayFolder="" measureGroup="customers" count="0" hidden="1">
+      <extLst>
+        <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{B97F6D7D-B522-45F9-BDA1-12C45D357490}">
+          <x15:cacheHierarchy aggregatedColumn="13"/>
+        </ext>
+      </extLst>
+    </cacheHierarchy>
+  </cacheHierarchies>
+  <kpis count="0"/>
+  <dimensions count="3">
+    <dimension name="calls" uniqueName="[calls]" caption="calls"/>
+    <dimension name="customers" uniqueName="[customers]" caption="customers"/>
+    <dimension measure="1" name="Measures" uniqueName="[Measures]" caption="Measures"/>
+  </dimensions>
+  <measureGroups count="2">
+    <measureGroup name="calls" caption="calls"/>
+    <measureGroup name="customers" caption="customers"/>
+  </measureGroups>
+  <maps count="3">
+    <map measureGroup="0" dimension="0"/>
+    <map measureGroup="0" dimension="1"/>
+    <map measureGroup="1" dimension="1"/>
+  </maps>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{725AE2AE-9491-48be-B2B4-4EB974FC3084}">
+      <x14:pivotCacheDefinition supportSubqueryNonVisual="1" supportSubqueryCalcMem="1" supportAddCalcMems="1"/>
+    </ext>
+  </extLst>
+</pivotCacheDefinition>
+</file>
+
+<file path=xl/pivotCache/pivotCacheDefinition8.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" saveData="0" refreshedBy="sivanagajyothi yedururu" refreshedDate="45755.942237615738" backgroundQuery="1" createdVersion="3" refreshedVersion="8" minRefreshableVersion="3" recordCount="0" supportSubquery="1" supportAdvancedDrill="1" xr:uid="{D57CF18B-F812-42BE-9712-7347525B42E3}">
   <cacheSource type="external" connectionId="2">
     <extLst>
@@ -13643,7 +13357,550 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{AAB53815-8D20-4469-8EC4-4352A86443FA}" name="weekly trend" cacheId="135" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" subtotalHiddenItems="1" itemPrintTitles="1" createdVersion="8" indent="0" multipleFieldFilters="0" chartFormat="23">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{D9E374A0-80E0-458F-B320-3A43586A0385}" name="PivotTable1" cacheId="33" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" multipleFieldFilters="0" chartFormat="10">
+  <location ref="D55:G60" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
+  <pivotFields count="3">
+    <pivotField axis="axisRow" allDrilled="1" showAll="0" dataSourceSort="1" defaultAttributeDrillState="1">
+      <items count="4">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField axis="axisCol" allDrilled="1" showAll="0" dataSourceSort="1" defaultAttributeDrillState="1">
+      <items count="3">
+        <item x="0"/>
+        <item x="1"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField dataField="1" showAll="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="0"/>
+  </rowFields>
+  <rowItems count="4">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colFields count="1">
+    <field x="1"/>
+  </colFields>
+  <colItems count="3">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </colItems>
+  <dataFields count="1">
+    <dataField fld="2" subtotal="count" baseField="0" baseItem="0"/>
+  </dataFields>
+  <chartFormats count="5">
+    <chartFormat chart="2" format="2" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="1" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="2" format="3" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="1" count="1" selected="0">
+            <x v="1"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="3" format="4" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="1" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="3" format="5" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="1" count="1" selected="0">
+            <x v="1"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="3" format="6">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="3">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="0" count="1" selected="0">
+            <x v="1"/>
+          </reference>
+          <reference field="1" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+  </chartFormats>
+  <pivotHierarchies count="27">
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+  </pivotHierarchies>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <rowHierarchiesUsage count="1">
+    <rowHierarchyUsage hierarchyUsage="15"/>
+  </rowHierarchiesUsage>
+  <colHierarchiesUsage count="1">
+    <colHierarchyUsage hierarchyUsage="13"/>
+  </colHierarchiesUsage>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" calculatedMembersInFilters="1" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{E67621CE-5B39-4880-91FE-76760E9C1902}">
+      <x15:pivotTableUISettings>
+        <x15:activeTabTopLevelEntity name="[customers]"/>
+        <x15:activeTabTopLevelEntity name="[calls]"/>
+      </x15:pivotTableUISettings>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{2C89DBDB-5792-4DE1-B0D8-F6BE6B3A85F2}" name="rep pivot" cacheId="19" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" subtotalHiddenItems="1" itemPrintTitles="1" createdVersion="8" indent="0" multipleFieldFilters="0">
+  <location ref="A11:E12" firstHeaderRow="0" firstDataRow="1" firstDataCol="0"/>
+  <pivotFields count="6">
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField allDrilled="1" showAll="0" dataSourceSort="1" defaultAttributeDrillState="1"/>
+  </pivotFields>
+  <rowItems count="1">
+    <i/>
+  </rowItems>
+  <colFields count="1">
+    <field x="-2"/>
+  </colFields>
+  <colItems count="5">
+    <i>
+      <x/>
+    </i>
+    <i i="1">
+      <x v="1"/>
+    </i>
+    <i i="2">
+      <x v="2"/>
+    </i>
+    <i i="3">
+      <x v="3"/>
+    </i>
+    <i i="4">
+      <x v="4"/>
+    </i>
+  </colItems>
+  <dataFields count="5">
+    <dataField fld="0" subtotal="count" baseField="0" baseItem="0"/>
+    <dataField fld="1" subtotal="count" baseField="0" baseItem="0"/>
+    <dataField fld="2" subtotal="count" baseField="0" baseItem="0"/>
+    <dataField fld="3" subtotal="count" baseField="0" baseItem="0"/>
+    <dataField fld="4" subtotal="count" baseField="0" baseItem="0"/>
+  </dataFields>
+  <pivotHierarchies count="27">
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy multipleItemSelectionAllowed="1" dragToData="1">
+      <members count="1" level="1">
+        <member name="[calls].[Representative].&amp;[R05]"/>
+      </members>
+    </pivotHierarchy>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+  </pivotHierarchies>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <colHierarchiesUsage count="1">
+    <colHierarchyUsage hierarchyUsage="-2"/>
+  </colHierarchiesUsage>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" calculatedMembersInFilters="1" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{E67621CE-5B39-4880-91FE-76760E9C1902}">
+      <x15:pivotTableUISettings sourceDataName="WorksheetConnection_excel_portfolioproject.xlsx!calls">
+        <x15:activeTabTopLevelEntity name="[calls]"/>
+      </x15:pivotTableUISettings>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{88456301-C695-4DCF-807F-7BCA00D1AD0A}" name="summary pivot" cacheId="20" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" multipleFieldFilters="0">
+  <location ref="A3:E4" firstHeaderRow="0" firstDataRow="1" firstDataCol="0"/>
+  <pivotFields count="5">
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField dataField="1" showAll="0"/>
+  </pivotFields>
+  <rowItems count="1">
+    <i/>
+  </rowItems>
+  <colFields count="1">
+    <field x="-2"/>
+  </colFields>
+  <colItems count="5">
+    <i>
+      <x/>
+    </i>
+    <i i="1">
+      <x v="1"/>
+    </i>
+    <i i="2">
+      <x v="2"/>
+    </i>
+    <i i="3">
+      <x v="3"/>
+    </i>
+    <i i="4">
+      <x v="4"/>
+    </i>
+  </colItems>
+  <dataFields count="5">
+    <dataField fld="0" subtotal="count" baseField="0" baseItem="0"/>
+    <dataField fld="1" subtotal="count" baseField="0" baseItem="0"/>
+    <dataField fld="2" subtotal="count" baseField="0" baseItem="0"/>
+    <dataField fld="3" subtotal="count" baseField="0" baseItem="0"/>
+    <dataField fld="4" subtotal="count" baseField="0" baseItem="0"/>
+  </dataFields>
+  <pivotHierarchies count="27">
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+  </pivotHierarchies>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <colHierarchiesUsage count="1">
+    <colHierarchyUsage hierarchyUsage="-2"/>
+  </colHierarchiesUsage>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" calculatedMembersInFilters="1" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{E67621CE-5B39-4880-91FE-76760E9C1902}">
+      <x15:pivotTableUISettings sourceDataName="WorksheetConnection_excel_portfolioproject.xlsx!calls">
+        <x15:activeTabTopLevelEntity name="[calls]"/>
+      </x15:pivotTableUISettings>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{D9FABC9E-27C8-4580-ADE9-CEF021B283CD}" name="selected_rep_pivot" cacheId="21" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" multipleFieldFilters="0">
+  <location ref="A58:A60" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <pivotFields count="1">
+    <pivotField axis="axisRow" allDrilled="1" showAll="0" dataSourceSort="1" defaultAttributeDrillState="1">
+      <items count="2">
+        <item s="1" x="0"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="0"/>
+  </rowFields>
+  <rowItems count="2">
+    <i>
+      <x/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <formats count="1">
+    <format dxfId="14">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="1">
+          <reference field="0" count="0"/>
+        </references>
+      </pivotArea>
+    </format>
+  </formats>
+  <pivotHierarchies count="27">
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy multipleItemSelectionAllowed="1" dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+  </pivotHierarchies>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <rowHierarchiesUsage count="1">
+    <rowHierarchyUsage hierarchyUsage="3"/>
+  </rowHierarchiesUsage>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" calculatedMembersInFilters="1" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{E67621CE-5B39-4880-91FE-76760E9C1902}">
+      <x15:pivotTableUISettings>
+        <x15:activeTabTopLevelEntity name="[calls]"/>
+      </x15:pivotTableUISettings>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable5.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{B1BDC753-0EA3-48CF-831C-1EBE078F2F26}" name="reps pivot" cacheId="22" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" multipleFieldFilters="0" chartFormat="5">
+  <location ref="A43:C49" firstHeaderRow="0" firstDataRow="1" firstDataCol="1"/>
+  <pivotFields count="3">
+    <pivotField axis="axisRow" allDrilled="1" showAll="0" dataSourceSort="1" defaultAttributeDrillState="1">
+      <items count="6">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField dataField="1" showAll="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="0"/>
+  </rowFields>
+  <rowItems count="6">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i>
+      <x v="4"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colFields count="1">
+    <field x="-2"/>
+  </colFields>
+  <colItems count="2">
+    <i>
+      <x/>
+    </i>
+    <i i="1">
+      <x v="1"/>
+    </i>
+  </colItems>
+  <dataFields count="2">
+    <dataField fld="1" subtotal="count" baseField="0" baseItem="0"/>
+    <dataField fld="2" subtotal="count" baseField="0" baseItem="0"/>
+  </dataFields>
+  <pivotHierarchies count="27">
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+  </pivotHierarchies>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <rowHierarchiesUsage count="1">
+    <rowHierarchyUsage hierarchyUsage="3"/>
+  </rowHierarchiesUsage>
+  <colHierarchiesUsage count="1">
+    <colHierarchyUsage hierarchyUsage="-2"/>
+  </colHierarchiesUsage>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" calculatedMembersInFilters="1" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{E67621CE-5B39-4880-91FE-76760E9C1902}">
+      <x15:pivotTableUISettings>
+        <x15:activeTabTopLevelEntity name="[calls]"/>
+      </x15:pivotTableUISettings>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable6.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{AAB53815-8D20-4469-8EC4-4352A86443FA}" name="weekly trend" cacheId="23" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" subtotalHiddenItems="1" itemPrintTitles="1" createdVersion="8" indent="0" multipleFieldFilters="0" chartFormat="23">
   <location ref="E19:F27" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="3">
     <pivotField allDrilled="1" showAll="0" dataSourceSort="1" defaultAttributeDrillState="1"/>
@@ -13725,7 +13982,7 @@
       </pivotArea>
     </chartFormat>
   </chartFormats>
-  <pivotHierarchies count="26">
+  <pivotHierarchies count="27">
     <pivotHierarchy dragToData="1"/>
     <pivotHierarchy dragToData="1"/>
     <pivotHierarchy dragToData="1"/>
@@ -13756,6 +14013,7 @@
     <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
     <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
     <pivotHierarchy dragToData="1" caption="call count1"/>
+    <pivotHierarchy dragToData="1"/>
   </pivotHierarchies>
   <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
   <rowHierarchiesUsage count="1">
@@ -13777,8 +14035,8 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{0CE4B034-F5D3-48CB-8B96-4EDB0797DC50}" name="month trend" cacheId="132" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" subtotalHiddenItems="1" itemPrintTitles="1" createdVersion="8" indent="0" multipleFieldFilters="0" chartFormat="11">
+<file path=xl/pivotTables/pivotTable7.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{0CE4B034-F5D3-48CB-8B96-4EDB0797DC50}" name="month trend" cacheId="24" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" subtotalHiddenItems="1" itemPrintTitles="1" createdVersion="8" indent="0" multipleFieldFilters="0" chartFormat="11">
   <location ref="A19:C32" firstHeaderRow="0" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="5">
     <pivotField allDrilled="1" showAll="0" dataSourceSort="1" defaultAttributeDrillState="1"/>
@@ -14045,7 +14303,7 @@
       </pivotArea>
     </chartFormat>
   </chartFormats>
-  <pivotHierarchies count="26">
+  <pivotHierarchies count="27">
     <pivotHierarchy dragToData="1"/>
     <pivotHierarchy dragToData="1"/>
     <pivotHierarchy dragToData="1"/>
@@ -14076,6 +14334,7 @@
     <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
     <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
     <pivotHierarchy dragToData="1" caption="call count1"/>
+    <pivotHierarchy dragToData="1"/>
   </pivotHierarchies>
   <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
   <rowHierarchiesUsage count="2">
@@ -14091,372 +14350,6 @@
     </ext>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{E67621CE-5B39-4880-91FE-76760E9C1902}">
       <x15:pivotTableUISettings sourceDataName="WorksheetConnection_excel_portfolioproject.xlsx!calls">
-        <x15:activeTabTopLevelEntity name="[calls]"/>
-      </x15:pivotTableUISettings>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{2C89DBDB-5792-4DE1-B0D8-F6BE6B3A85F2}" name="rep pivot" cacheId="129" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" subtotalHiddenItems="1" itemPrintTitles="1" createdVersion="8" indent="0" multipleFieldFilters="0">
-  <location ref="A11:E12" firstHeaderRow="0" firstDataRow="1" firstDataCol="0"/>
-  <pivotFields count="6">
-    <pivotField dataField="1" showAll="0"/>
-    <pivotField dataField="1" showAll="0"/>
-    <pivotField dataField="1" showAll="0"/>
-    <pivotField dataField="1" showAll="0"/>
-    <pivotField dataField="1" showAll="0"/>
-    <pivotField allDrilled="1" showAll="0" dataSourceSort="1" defaultAttributeDrillState="1"/>
-  </pivotFields>
-  <rowItems count="1">
-    <i/>
-  </rowItems>
-  <colFields count="1">
-    <field x="-2"/>
-  </colFields>
-  <colItems count="5">
-    <i>
-      <x/>
-    </i>
-    <i i="1">
-      <x v="1"/>
-    </i>
-    <i i="2">
-      <x v="2"/>
-    </i>
-    <i i="3">
-      <x v="3"/>
-    </i>
-    <i i="4">
-      <x v="4"/>
-    </i>
-  </colItems>
-  <dataFields count="5">
-    <dataField fld="0" subtotal="count" baseField="0" baseItem="0"/>
-    <dataField fld="1" subtotal="count" baseField="0" baseItem="0"/>
-    <dataField fld="2" subtotal="count" baseField="0" baseItem="0"/>
-    <dataField fld="3" subtotal="count" baseField="0" baseItem="0"/>
-    <dataField fld="4" subtotal="count" baseField="0" baseItem="0"/>
-  </dataFields>
-  <pivotHierarchies count="26">
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy multipleItemSelectionAllowed="1" dragToData="1">
-      <members count="1" level="1">
-        <member name="[calls].[Representative].&amp;[R05]"/>
-      </members>
-    </pivotHierarchy>
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
-    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
-    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
-    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
-    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
-    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
-    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
-    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
-    <pivotHierarchy dragToData="1"/>
-  </pivotHierarchies>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <colHierarchiesUsage count="1">
-    <colHierarchyUsage hierarchyUsage="-2"/>
-  </colHierarchiesUsage>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" calculatedMembersInFilters="1" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{E67621CE-5B39-4880-91FE-76760E9C1902}">
-      <x15:pivotTableUISettings sourceDataName="WorksheetConnection_excel_portfolioproject.xlsx!calls">
-        <x15:activeTabTopLevelEntity name="[calls]"/>
-      </x15:pivotTableUISettings>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{88456301-C695-4DCF-807F-7BCA00D1AD0A}" name="summary pivot" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" multipleFieldFilters="0">
-  <location ref="A3:E4" firstHeaderRow="0" firstDataRow="1" firstDataCol="0"/>
-  <pivotFields count="5">
-    <pivotField dataField="1" showAll="0"/>
-    <pivotField dataField="1" showAll="0"/>
-    <pivotField dataField="1" showAll="0"/>
-    <pivotField dataField="1" showAll="0"/>
-    <pivotField dataField="1" showAll="0"/>
-  </pivotFields>
-  <rowItems count="1">
-    <i/>
-  </rowItems>
-  <colFields count="1">
-    <field x="-2"/>
-  </colFields>
-  <colItems count="5">
-    <i>
-      <x/>
-    </i>
-    <i i="1">
-      <x v="1"/>
-    </i>
-    <i i="2">
-      <x v="2"/>
-    </i>
-    <i i="3">
-      <x v="3"/>
-    </i>
-    <i i="4">
-      <x v="4"/>
-    </i>
-  </colItems>
-  <dataFields count="5">
-    <dataField fld="0" subtotal="count" baseField="0" baseItem="0"/>
-    <dataField fld="1" subtotal="count" baseField="0" baseItem="0"/>
-    <dataField fld="2" subtotal="count" baseField="0" baseItem="0"/>
-    <dataField fld="3" subtotal="count" baseField="0" baseItem="0"/>
-    <dataField fld="4" subtotal="count" baseField="0" baseItem="0"/>
-  </dataFields>
-  <pivotHierarchies count="26">
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
-    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
-    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
-    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
-    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
-    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
-    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
-    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
-    <pivotHierarchy dragToData="1"/>
-  </pivotHierarchies>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <colHierarchiesUsage count="1">
-    <colHierarchyUsage hierarchyUsage="-2"/>
-  </colHierarchiesUsage>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" calculatedMembersInFilters="1" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{E67621CE-5B39-4880-91FE-76760E9C1902}">
-      <x15:pivotTableUISettings sourceDataName="WorksheetConnection_excel_portfolioproject.xlsx!calls">
-        <x15:activeTabTopLevelEntity name="[calls]"/>
-      </x15:pivotTableUISettings>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable5.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{D9FABC9E-27C8-4580-ADE9-CEF021B283CD}" name="selected_rep_pivot" cacheId="138" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" multipleFieldFilters="0">
-  <location ref="A58:A60" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
-  <pivotFields count="1">
-    <pivotField axis="axisRow" allDrilled="1" showAll="0" dataSourceSort="1" defaultAttributeDrillState="1">
-      <items count="2">
-        <item s="1" x="0"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-  </pivotFields>
-  <rowFields count="1">
-    <field x="0"/>
-  </rowFields>
-  <rowItems count="2">
-    <i>
-      <x/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <formats count="1">
-    <format dxfId="14">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="1">
-          <reference field="0" count="0"/>
-        </references>
-      </pivotArea>
-    </format>
-  </formats>
-  <pivotHierarchies count="26">
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy multipleItemSelectionAllowed="1" dragToData="1"/>
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
-    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
-    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
-    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
-    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
-    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
-    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
-    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
-    <pivotHierarchy dragToData="1"/>
-  </pivotHierarchies>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <rowHierarchiesUsage count="1">
-    <rowHierarchyUsage hierarchyUsage="3"/>
-  </rowHierarchiesUsage>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" calculatedMembersInFilters="1" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{E67621CE-5B39-4880-91FE-76760E9C1902}">
-      <x15:pivotTableUISettings>
-        <x15:activeTabTopLevelEntity name="[calls]"/>
-      </x15:pivotTableUISettings>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable6.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{B1BDC753-0EA3-48CF-831C-1EBE078F2F26}" name="reps pivot" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" multipleFieldFilters="0" chartFormat="5">
-  <location ref="A43:C49" firstHeaderRow="0" firstDataRow="1" firstDataCol="1"/>
-  <pivotFields count="3">
-    <pivotField axis="axisRow" allDrilled="1" showAll="0" dataSourceSort="1" defaultAttributeDrillState="1">
-      <items count="6">
-        <item x="0"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item x="3"/>
-        <item x="4"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField dataField="1" showAll="0"/>
-    <pivotField dataField="1" showAll="0"/>
-  </pivotFields>
-  <rowFields count="1">
-    <field x="0"/>
-  </rowFields>
-  <rowItems count="6">
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="2"/>
-    </i>
-    <i>
-      <x v="3"/>
-    </i>
-    <i>
-      <x v="4"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colFields count="1">
-    <field x="-2"/>
-  </colFields>
-  <colItems count="2">
-    <i>
-      <x/>
-    </i>
-    <i i="1">
-      <x v="1"/>
-    </i>
-  </colItems>
-  <dataFields count="2">
-    <dataField fld="1" subtotal="count" baseField="0" baseItem="0"/>
-    <dataField fld="2" subtotal="count" baseField="0" baseItem="0"/>
-  </dataFields>
-  <pivotHierarchies count="26">
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
-    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
-    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
-    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
-    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
-    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
-    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
-    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
-    <pivotHierarchy dragToData="1"/>
-  </pivotHierarchies>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <rowHierarchiesUsage count="1">
-    <rowHierarchyUsage hierarchyUsage="3"/>
-  </rowHierarchiesUsage>
-  <colHierarchiesUsage count="1">
-    <colHierarchyUsage hierarchyUsage="-2"/>
-  </colHierarchiesUsage>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" calculatedMembersInFilters="1" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{E67621CE-5B39-4880-91FE-76760E9C1902}">
-      <x15:pivotTableUISettings>
         <x15:activeTabTopLevelEntity name="[calls]"/>
       </x15:pivotTableUISettings>
     </ext>
@@ -14810,7 +14703,7 @@
 
 <file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
 <wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
-  <wetp:taskpane dockstate="right" visibility="1" width="438" row="7">
+  <wetp:taskpane dockstate="right" visibility="1" width="493" row="6">
     <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </wetp:taskpane>
 </wetp:taskpanes>
@@ -22535,10 +22428,10 @@
     <col min="1" max="1" width="13.33203125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="10.44140625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="9.44140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9.6640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.33203125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="9.44140625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="10.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="16.5546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.6640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
@@ -22596,7 +22489,7 @@
       <c r="A12" s="21">
         <v>200</v>
       </c>
-      <c r="B12" s="30">
+      <c r="B12" s="22">
         <v>20104</v>
       </c>
       <c r="C12" s="23">
@@ -22630,7 +22523,7 @@
       <c r="A20" s="27" t="s">
         <v>1073</v>
       </c>
-      <c r="B20" s="31">
+      <c r="B20">
         <v>21</v>
       </c>
       <c r="C20" s="21">
@@ -22647,7 +22540,7 @@
       <c r="A21" s="27" t="s">
         <v>1074</v>
       </c>
-      <c r="B21" s="31">
+      <c r="B21">
         <v>18</v>
       </c>
       <c r="C21" s="21">
@@ -22664,7 +22557,7 @@
       <c r="A22" s="27" t="s">
         <v>1075</v>
       </c>
-      <c r="B22" s="31">
+      <c r="B22">
         <v>31</v>
       </c>
       <c r="C22" s="21">
@@ -22681,7 +22574,7 @@
       <c r="A23" s="27" t="s">
         <v>1076</v>
       </c>
-      <c r="B23" s="31">
+      <c r="B23">
         <v>20</v>
       </c>
       <c r="C23" s="21">
@@ -22698,7 +22591,7 @@
       <c r="A24" s="27" t="s">
         <v>1077</v>
       </c>
-      <c r="B24" s="31">
+      <c r="B24">
         <v>8</v>
       </c>
       <c r="C24" s="21">
@@ -22715,7 +22608,7 @@
       <c r="A25" s="27" t="s">
         <v>1078</v>
       </c>
-      <c r="B25" s="31">
+      <c r="B25">
         <v>12</v>
       </c>
       <c r="C25" s="21">
@@ -22732,7 +22625,7 @@
       <c r="A26" s="27" t="s">
         <v>1079</v>
       </c>
-      <c r="B26" s="31">
+      <c r="B26">
         <v>12</v>
       </c>
       <c r="C26" s="21">
@@ -22749,7 +22642,7 @@
       <c r="A27" s="27" t="s">
         <v>1080</v>
       </c>
-      <c r="B27" s="31">
+      <c r="B27">
         <v>7</v>
       </c>
       <c r="C27" s="21">
@@ -22766,7 +22659,7 @@
       <c r="A28" s="27" t="s">
         <v>1081</v>
       </c>
-      <c r="B28" s="31">
+      <c r="B28">
         <v>20</v>
       </c>
       <c r="C28" s="21">
@@ -22777,7 +22670,7 @@
       <c r="A29" s="27" t="s">
         <v>1082</v>
       </c>
-      <c r="B29" s="31">
+      <c r="B29">
         <v>24</v>
       </c>
       <c r="C29" s="21">
@@ -22788,7 +22681,7 @@
       <c r="A30" s="27" t="s">
         <v>1083</v>
       </c>
-      <c r="B30" s="31">
+      <c r="B30">
         <v>12</v>
       </c>
       <c r="C30" s="21">
@@ -22799,7 +22692,7 @@
       <c r="A31" s="27" t="s">
         <v>1084</v>
       </c>
-      <c r="B31" s="31">
+      <c r="B31">
         <v>15</v>
       </c>
       <c r="C31" s="21">
@@ -22810,7 +22703,7 @@
       <c r="A32" s="27" t="s">
         <v>1072</v>
       </c>
-      <c r="B32" s="31">
+      <c r="B32">
         <v>200</v>
       </c>
       <c r="C32" s="21">
@@ -23004,7 +22897,7 @@
         <v>20104</v>
       </c>
     </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A49" s="27" t="s">
         <v>1072</v>
       </c>
@@ -23015,29 +22908,101 @@
         <v>96623</v>
       </c>
     </row>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="D55" s="24" t="s">
+        <v>1042</v>
+      </c>
+      <c r="E55" s="24" t="s">
+        <v>1093</v>
+      </c>
+    </row>
+    <row r="56" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="D56" s="24" t="s">
+        <v>1071</v>
+      </c>
+      <c r="E56" t="s">
+        <v>999</v>
+      </c>
+      <c r="F56" t="s">
+        <v>998</v>
+      </c>
+      <c r="G56" t="s">
+        <v>1072</v>
+      </c>
+    </row>
+    <row r="57" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="D57" s="27" t="s">
+        <v>1002</v>
+      </c>
+      <c r="E57" s="21">
+        <v>144</v>
+      </c>
+      <c r="F57" s="21">
+        <v>132</v>
+      </c>
+      <c r="G57" s="21">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="58" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A58" s="24" t="s">
         <v>1071</v>
       </c>
-    </row>
-    <row r="59" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D58" s="27" t="s">
+        <v>1001</v>
+      </c>
+      <c r="E58" s="21">
+        <v>326</v>
+      </c>
+      <c r="F58" s="21">
+        <v>63</v>
+      </c>
+      <c r="G58" s="21">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="59" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A59" s="28" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="60" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D59" s="27" t="s">
+        <v>1000</v>
+      </c>
+      <c r="E59" s="21">
+        <v>129</v>
+      </c>
+      <c r="F59" s="21">
+        <v>206</v>
+      </c>
+      <c r="G59" s="21">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="60" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A60" s="27" t="s">
         <v>1072</v>
       </c>
+      <c r="D60" s="27" t="s">
+        <v>1072</v>
+      </c>
+      <c r="E60" s="21">
+        <v>599</v>
+      </c>
+      <c r="F60" s="21">
+        <v>401</v>
+      </c>
+      <c r="G60" s="21">
+        <v>1000</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId7"/>
-  <drawing r:id="rId8"/>
+  <pageSetup orientation="portrait" r:id="rId8"/>
+  <drawing r:id="rId9"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{A8765BA9-456A-4dab-B4F3-ACF838C121DE}">
       <x14:slicerList>
-        <x14:slicer r:id="rId9"/>
+        <x14:slicer r:id="rId10"/>
       </x14:slicerList>
     </ext>
   </extLst>

</xml_diff>